<commit_message>
docs: clean up model-derived metadata text
</commit_message>
<xml_diff>
--- a/Documents/Health-RI_v2.1.0-for-FDP.xlsx
+++ b/Documents/Health-RI_v2.1.0-for-FDP.xlsx
@@ -179,7 +179,7 @@
         <scheme val="major"/>
       </rPr>
       <t xml:space="preserve">This property points to a contact point that can answer questions about the dataset. Details on how to describe these are provided under class vcard:Kind.
-Whenever possible, use a </t>
+Whenever possible, use </t>
     </r>
     <r>
       <rPr>
@@ -198,7 +198,7 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t xml:space="preserve"> (for example from a department) instead of contact information of an individual.</t>
+      <t xml:space="preserve"> (for example from a department) instead of the contact information of an individual.</t>
     </r>
   </si>
   <si>
@@ -227,7 +227,7 @@
   </si>
   <si>
     <t>The creator is the entity responsible for making the resource. According to Dutch databank and copyright law, this is in most cases the organisation / employer bearing investment risk, instead of an individual (e.g. individual researcher). Therefore, in many cases, this might be the same Agent as the dct:publisher, being the organisation (not a department or subdivision of the organisation) where the catalogue was created.
-In case there are multiple (collaborating) organisation involved in data creation, all of them can be stated as dct:creator, as the model allows more than one creator.
+In case there are multiple (collaborating) organisations involved in data creation, all of them can be stated as dct:creator, as the model allows more than one creator.
 Note that the Health-RI model diverges from DCAT-AP NL here, which reduces the maximum number of creators to 1. The Health-RI model allows the specification of multiple creators of a catalogue.</t>
   </si>
   <si>
@@ -551,7 +551,7 @@
     <t>access rights</t>
   </si>
   <si>
-    <t>Information about who access the resource or an indication of its security status.</t>
+    <t>Information about who can access the resource or an indication of its security status.</t>
   </si>
   <si>
     <t>dct:accessRights</t>
@@ -560,10 +560,10 @@
     <t>http://publications.europa.eu/resource/authority/access-right</t>
   </si>
   <si>
-    <t>Information that indicates whether the Dataset is publicly accessible, has access restrictions or is not public. It is foreseen that one of the three options have to be used: public, restricted, non-public.
+    <t>Information that indicates whether the Dataset is publicly accessible, has access restrictions or is not public. It is foreseen that one of the three options has to be used: public, restricted, non-public.
     Open Data (Public): The dataset is available under general open data rules, such as those covered by the High Value Datasets Implementing Regulation.
     Protected Data (Restricted): The dataset contains protected data and is accessible only under specific conditions, as outlined in regulations like the Data Governance Act.
-    Sensitive Data (Non public): The dataset includes resources that may contain sensitive or personal information, falling under regulations such as the EHDS Regulation.
+    Sensitive Data (Non-public): The dataset includes resources that may contain sensitive or personal information, falling under regulations such as the EHDS Regulation.
 Since most data contain personal information, these datasets will need to take the value 'non-public' for the access rights property.</t>
   </si>
   <si>
@@ -579,7 +579,7 @@
     <t>healthdcatap:analytics</t>
   </si>
   <si>
-    <t>Publishers are encouraged to provide URLs pointing to document repositories where users can access or request associated resources such as technical reports of the dataset, quality measurements, usability indicators,... Note that HealthDCAT-AP mentions also API endpoints or analytics services, but these would not be Distriutions but rather DatasetServices.</t>
+    <t>Publishers are encouraged to provide URLs pointing to document repositories where users can access or request associated resources such as technical reports of the dataset, quality measurements, usability indicators, etc. Note that HealthDCAT-AP also mentions API endpoints or analytics services, but these would not be Distributions but rather DatasetServices.</t>
   </si>
   <si>
     <t>dcat:Distribution</t>
@@ -637,8 +637,8 @@
   </si>
   <si>
     <t>The creator (of the dataset) is the entity responsible for making the resource. According to Dutch databank and copyright law, this is in most cases the organisation / employer bearing investment risk, instead of an individual (e.g. individual researcher). Therefore, in many cases, this might be the same Agent as the dct:publisher, being the organisation (not a department or subdivision of the organisation) where the dataset was created.
-In case there are multiple (collaborating) organisation involved in data creation, all of them can be stated as dct:creator, as the model allows more than one creator.
-In case you wish to credit other contributors to the dataset, you can use the prov:qualifiedAttribution property. This could be useful if you wish to indicate, for example, the funding organisation(s), collaborating organosation(s) or name specific individuals (e.g., principal investigator) involved in creation or managing of the dataset.</t>
+In case there are multiple (collaborating) organisations involved in data creation, all of them can be stated as dct:creator, as the model allows more than one creator.
+In case you wish to credit other contributors to the dataset, you can use the prov:qualifiedAttribution property. This could be useful if you wish to indicate, for example, the funding organisation(s), collaborating organisation(s) or name specific individuals (e.g., principal investigator) involved in creating or managing the dataset.</t>
   </si>
   <si>
     <t>custom:creator_</t>
@@ -696,7 +696,7 @@
     <t>custom:frequency</t>
   </si>
   <si>
-    <t>The EU Vocabularies Name Authority Lists must be used for continents, countries and places that are in those lists; if a particular location is not in one of the mentioned Named Authority Lists, Geonames URIs must be used. For districts or neighbourhoods in NL, the Dutch vocab can be used. However, it might in many cases be desirable to keep the geographical coverage broader (eg. indicating that NL is covered), to not expose detailed information of subject's locations.</t>
+    <t>The EU Vocabularies Name Authority Lists must be used for continents, countries and places that are in those lists; if a particular location is not in one of the mentioned Named Authority Lists, Geonames URIs must be used. For districts or neighbourhoods in NL, the Dutch vocab can be used. However, it might in many cases be desirable to keep the geographical coverage broader (e.g. indicating that NL is covered), to avoid exposing detailed information about subjects' locations.</t>
   </si>
   <si>
     <t>has version</t>
@@ -738,7 +738,7 @@
     <t>dct:identifier</t>
   </si>
   <si>
-    <t>Current status: Health-RI is currently working on a strategy for persistant identifiers for, among other things, datasets. Until a solid solution has been found, we propose the following temporary solution:
+    <t>Current status: Health-RI is currently working on a strategy for persistent identifiers for, among other things, datasets. Until a solid solution has been found, we propose the following temporary solution:
 If your data is published in a repository, fill in with the provided DOI (Example: https://doi.org/10.34894/ZLOYOJ). If not, use the identifier of the dataset as generated in the FAIR data point (FDP). Ensure that metadata is updated if your situation changes.</t>
   </si>
   <si>
@@ -1322,7 +1322,7 @@
 Wikidata: https://www.wikidata.org/wiki/Wikidata:Main_Page</t>
   </si>
   <si>
-    <t>Specify the entity (person or organization) by providing an identifier. We recommend using an ORCID identifier for a person or ROR identifier for organization. Dutch governmenta organization are listed in TOOI. If these are not available, you can use ISNI, or Wikidata or any other identifier you may have. If you have multiple identifiers, you should provide them all.</t>
+    <t>Specify the entity (person or organization) by providing an identifier. We recommend using an ORCID identifier for a person or ROR identifier for an organization. Dutch government organizations are listed in TOOI. If these are not available, you can use ISNI, or Wikidata or any other identifier you may have. If you have multiple identifiers, you should provide them all.</t>
   </si>
   <si>
     <t>HRI v1</t>
@@ -1433,7 +1433,7 @@
     <t>vcard:hasURL</t>
   </si>
   <si>
-    <t>A webpage that either allows to make contact (i.e. a webform) or the information contains how to get into contact.</t>
+    <t>A webpage that either allows contact (i.e. a web form) or contains information on how to make contact.</t>
   </si>
   <si>
     <t>custom:{property}_url</t>
@@ -1520,7 +1520,7 @@
     <t>dcat:byteSize</t>
   </si>
   <si>
-    <t>Describes the size of the distribution (the actual file) in bytes, and is therefore expressed as a non-negative integer. If the actual size is not know, it can be estimated.</t>
+    <t>Describes the size of the distribution (the actual file) in bytes, and is therefore expressed as a non-negative integer. If the actual size is not known, it can be estimated.</t>
   </si>
   <si>
     <t>xsd:nonNegativeInteger</t>
@@ -1637,7 +1637,7 @@
         <scheme val="major"/>
       </rPr>
       <t xml:space="preserve"> used in the Distribution, indicated with a value from the EU controlled vocabulary. Not all distributions might have a language, for example imaging data.
-Note that here the Health-RI model diverges from DCAT-AP NL, which allows maximum of 1 languages per Distribution. The Health-RI model allows multiple languages in the same Distribution.</t>
+Note that here the Health-RI model diverges from DCAT-AP NL, which allows a maximum of 1 language per Distribution. The Health-RI model allows multiple languages in the same Distribution.</t>
     </r>
   </si>
   <si>
@@ -1674,7 +1674,7 @@
     <t>dcat:mediaType</t>
   </si>
   <si>
-    <t>Use the specified vocabularies, prioritizing IANA media types whenever possible. If unavailable, consider other ontologies, such as ZonMw generic terms, to descibe the format.
+    <t>Use the specified vocabularies, prioritizing IANA media types whenever possible. If unavailable, consider other ontologies, such as ZonMw generic terms, to describe the format.
 Example: https://www.iana.org/assignments/media-types/text/csv (for csv)
 If IANA media types do not sufficiently describe the format, use "format" to describe it in more detail.</t>
   </si>
@@ -1758,7 +1758,7 @@
     <t>data_series::coverage</t>
   </si>
   <si>
-    <t>This is not equal to the most recent modified dataset in the collection of the dataset series.</t>
+    <t>This is not equal to the most recently modified dataset in the collection of the dataset series.</t>
   </si>
   <si>
     <t xml:space="preserve">The publisher of the dataset series may not be the publisher of all datasets.  E.g. a digital archive could take over the publishing of older datasets in the series. </t>
@@ -1773,7 +1773,7 @@
     <t>data_series:issued</t>
   </si>
   <si>
-    <t>When temporal coverage is a dimension in the dataset series then the temporal coverage of each dataset in the collection should be part of the temporal coverage. In that case, an open ended value is recommended, e.g. after 2012.</t>
+    <t>When temporal coverage is a dimension in the dataset series then the temporal coverage of each dataset in the collection should be part of the temporal coverage. In that case, an open-ended value is recommended, e.g. after 2012.</t>
   </si>
   <si>
     <t>data_series::temporal</t>
@@ -1834,7 +1834,7 @@
     <t>application profile</t>
   </si>
   <si>
-    <t>The standards referred here SHOULD describe the Data Service and not the data it serves. The latter is provided by the dataset with which this Data Service is connected. For instance the data service adheres to the OGC WFS API standard, while the associated dataset adheres to the INSPIRE Address data model.</t>
+    <t>The standards referred to here SHOULD describe the Data Service and not the data it serves. The latter is provided by the dataset with which this Data Service is connected. For instance, the data service adheres to the OGC WFS API standard, while the associated dataset adheres to the INSPIRE Address data model.</t>
   </si>
   <si>
     <t>Briefly describe the data service provided. You can repeat this description in multiple languages. Example: A data service that provides API access to real-time electrocardiogram (ECG) monitoring data for clinical research applications.</t>
@@ -2121,7 +2121,7 @@
     <t>agent</t>
   </si>
   <si>
-    <t>The prov:agent property references an prov:Agent which influenced a resource.</t>
+    <t>The prov:agent property references a prov:Agent which influenced a resource.</t>
   </si>
   <si>
     <t>prov:agent</t>
@@ -2444,7 +2444,7 @@
     <t>checksum value</t>
   </si>
   <si>
-    <t>The checksumValue property provides a lower case hexidecimal encoded digest value produced using a specific algorithm.</t>
+    <t>The checksumValue property provides a lowercase hexadecimal-encoded digest value produced using a specific algorithm.</t>
   </si>
   <si>
     <t>spdx:checksumValue</t>
@@ -2479,12 +2479,12 @@
   </si>
   <si>
     <t>The legal basis can be provided as a value from the dpv taxonomy (see Controlled vocabulary column).
-While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property described the legal basis for initial collection and processing of (personal) data.
+While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property describes the legal basis for initial collection and processing of (personal) data.
 This property should always be filled if the dataset contains personal data and the applicable legislation is GDPR.
 Example value for this property could be: dpv:Consent</t>
   </si>
   <si>
-    <t>One (or many) categoiesy or sub-categories of the purposes can be chosen from the taxonomy provided by dpv (see controlled vocabulary column). Try to be as specific as possible.
+    <t>One (or many) categories or sub-categories of the purposes can be chosen from the taxonomy provided by dpv (see controlled vocabulary column). Try to be as specific as possible.
 Example value could be: dpv:ResearchAndDevelopment.</t>
   </si>
   <si>
@@ -2644,7 +2644,7 @@
     <t xml:space="preserve">A keyword or tag describing the table.	</t>
   </si>
   <si>
-    <t>Variable (column) defines metadata about one field in the CSV file.</t>
+    <t>A variable (column) defines metadata about one field in the CSV file.</t>
   </si>
   <si>
     <t>csvw:url</t>
@@ -2665,7 +2665,7 @@
     <t>Provides a set of keywords to support search and discovery of the table.</t>
   </si>
   <si>
-    <t>Each variable (column) node defines characteristics such as name, title, datatype, etc., for one column of the CSV. Should be either a blank node or IRI referring to a csvw:Column.</t>
+    <t>Each variable (column) node defines characteristics such as name, title, datatype, etc., for one column of the CSV. It should be either a blank node or an IRI referring to a csvw:Column.</t>
   </si>
   <si>
     <t>csvw:Column</t>
@@ -2680,10 +2680,10 @@
     <t>property URL</t>
   </si>
   <si>
-    <t>A Technical name given to the Variable as it appears in the CSV file.</t>
-  </si>
-  <si>
-    <t>A Human-readable name given to the Variable.</t>
+    <t>A technical name given to the Variable as it appears in the CSV file.</t>
+  </si>
+  <si>
+    <t>A human-readable name given to the Variable.</t>
   </si>
   <si>
     <t>Variable description.</t>
@@ -3363,7 +3363,7 @@
     </r>
   </si>
   <si>
-    <t>Information about how the data was collected, including methodologies, tools, and protocols used, this property can be repeated for different versions of the provenance (e.g. the provenance in different languages).
+    <t>Information about how the data was collected, including methodologies, tools, and protocols used. This property can be repeated for different versions of the provenance (e.g. the provenance in different languages).
 This is where the collection-method statements not captured by dedicated properties can be listed.</t>
   </si>
   <si>
@@ -3422,7 +3422,7 @@
         <scheme val="major"/>
       </rPr>
       <t>: The use of wikidata URIs will be replaced with the terms from a controlled vocabulary in the next major release.
-This property provides informatio on which coding systems are in use inside your dataset. For this, wikidata URIs must be used.</t>
+This property provides information on which coding systems are in use in your dataset. For this, wikidata URIs must be used.</t>
     </r>
   </si>
   <si>
@@ -3505,12 +3505,12 @@
     </r>
   </si>
   <si>
-    <t>A statement that concerns all rights not addressed in fields License or Access rights. In case of not open data (as specified in the dct:licence property), further agreements regarding data reuse (eg. Data Transfer Agreement, DTA,) should be stated in this property.
-The rights statement should be a free-text statement placed at an web-accessible location such that the value of this property is the IRI pointing to that statement.</t>
+    <t>A statement that concerns all rights not addressed in fields License or Access rights. In case of not open data (as specified in the dct:licence property), further agreements regarding data reuse (e.g. Data Transfer Agreement, DTA) should be stated in this property.
+The rights statement should be a free-text statement placed at a web-accessible location such that the value of this property is the IRI pointing to that statement.</t>
   </si>
   <si>
     <r>
-      <t xml:space="preserve">A email address via which contact can be made. This property </t>
+      <t xml:space="preserve">An email address via which contact can be made. This property </t>
     </r>
     <r>
       <rPr>

</xml_diff>

<commit_message>
fix(excel): apply 203 approved text corrections
</commit_message>
<xml_diff>
--- a/Documents/Health-RI_v2.1.0-for-FDP.xlsx
+++ b/Documents/Health-RI_v2.1.0-for-FDP.xlsx
@@ -78,7 +78,7 @@
     <t>Property URI</t>
   </si>
   <si>
-    <t>Controlled vocabluary (if applicable)</t>
+    <t>Controlled vocabulary (if applicable)</t>
   </si>
   <si>
     <t>Usage note</t>
@@ -138,16 +138,16 @@
     <t>custom:applicable_legislation</t>
   </si>
   <si>
-    <t>catalog</t>
-  </si>
-  <si>
-    <t>A catalog that is listed in the catalog.</t>
+    <t>catalogue</t>
+  </si>
+  <si>
+    <t>A catalogue that is listed in the catalogue.</t>
   </si>
   <si>
     <t>dcat:catalog</t>
   </si>
   <si>
-    <t>For certain research projects, multiple catalogs may need to be organized in a nested manner. This property serves to connect the different catalogs with each other.</t>
+    <t>For certain research projects, multiple catalogues may need to be organised in a nested manner. This property serves to connect the different catalogues with each other.</t>
   </si>
   <si>
     <t>dcat:Catalog</t>
@@ -165,7 +165,7 @@
     <t>contact point</t>
   </si>
   <si>
-    <t>Relevant contact information for the cataloged resource.</t>
+    <t>Relevant contact information for the catalogued resource.</t>
   </si>
   <si>
     <t>dcat:contactPoint</t>
@@ -178,7 +178,7 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t xml:space="preserve">This property points to a contact point that can answer questions about the dataset. Details on how to describe these are provided under class vcard:Kind.
+      <t xml:space="preserve">This property points to a contact point that can answer questions about the dataset. Details on how to describe these are provided under the vcard:Kind class.
 Whenever possible, use </t>
     </r>
     <r>
@@ -198,7 +198,7 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t xml:space="preserve"> (for example from a department) instead of the contact information of an individual.</t>
+      <t xml:space="preserve"> (for example, from a department) instead of the contact information of an individual.</t>
     </r>
   </si>
   <si>
@@ -214,7 +214,7 @@
     <t>custom:contact</t>
   </si>
   <si>
-    <t>fill in in 'Kind' tab</t>
+    <t>Enter the value on the 'Kind' tab.</t>
   </si>
   <si>
     <t>creator</t>
@@ -226,8 +226,8 @@
     <t>dct:creator</t>
   </si>
   <si>
-    <t>The creator is the entity responsible for making the resource. According to Dutch databank and copyright law, this is in most cases the organisation / employer bearing investment risk, instead of an individual (e.g. individual researcher). Therefore, in many cases, this might be the same Agent as the dct:publisher, being the organisation (not a department or subdivision of the organisation) where the catalogue was created.
-In case there are multiple (collaborating) organisations involved in data creation, all of them can be stated as dct:creator, as the model allows more than one creator.
+    <t>The creator is the entity responsible for making the resource. According to Dutch databank and copyright law, this is in most cases the organisation/employer bearing investment risk, instead of an individual (e.g. an individual researcher). Therefore, in many cases, this might be the same Agent as the dct:publisher: the organisation (not a department or subdivision of the organisation) where the catalogue was created.
+If there are multiple (collaborating) organisations involved in data creation, all of them can be stated as dct:creator, as the model allows more than one creator.
 Note that the Health-RI model diverges from DCAT-AP NL here, which reduces the maximum number of creators to 1. The Health-RI model allows the specification of multiple creators of a catalogue.</t>
   </si>
   <si>
@@ -237,19 +237,19 @@
     <t>custom:creator</t>
   </si>
   <si>
-    <t>fill in in 'Agent' tab</t>
+    <t>Enter the value on the 'Agent' tab.</t>
   </si>
   <si>
     <t>dataset</t>
   </si>
   <si>
-    <t>A dataset that is listed in the catalog.</t>
+    <t>A dataset that is listed in the catalogue.</t>
   </si>
   <si>
     <t>dcat:dataset</t>
   </si>
   <si>
-    <t>Each catalog contains one or more datasets. This property serves to link datasets to a catalogue. Therefore, a dataset is always contained inside a catalogue.</t>
+    <t>Each catalogue contains one or more datasets. This property serves to link datasets to a catalogue. Therefore, a dataset is always contained inside a catalogue.</t>
   </si>
   <si>
     <t>dcat:Dataset</t>
@@ -270,7 +270,7 @@
     <t>dct:description</t>
   </si>
   <si>
-    <t>Briefly describe the catalog and what it contains. You can repeat this in multiple languages.</t>
+    <t>Briefly describe the catalogue and what it contains. You can repeat this in multiple languages.</t>
   </si>
   <si>
     <t>rdfs:Literal</t>
@@ -291,7 +291,7 @@
     <t>EU Vocabularies Continents Named Authority List</t>
   </si>
   <si>
-    <t>The EU Vocabularies Name Authority Lists must be used for continents, countries and places that are in those lists; if a particular location is not in one of the mentioned Named Authority Lists, Geonames URIs must be used. For districts or neighbourhoods in NL, the Dutch vocab can be used.</t>
+    <t>The EU Vocabularies Named Authority Lists must be used for continents, countries and places that are in those lists; if a particular location is not in one of the mentioned Named Authority Lists, GeoNames URIs must be used. For districts or neighbourhoods in NL, the Dutch vocabulary can be used.</t>
   </si>
   <si>
     <t>dct:Location (IRI)</t>
@@ -306,7 +306,7 @@
     <t>EU Vocabularies Places Named Authority List</t>
   </si>
   <si>
-    <t>Geonames</t>
+    <t>GeoNames</t>
   </si>
   <si>
     <t>https://vocabs.cbs.nl/nl/</t>
@@ -322,10 +322,10 @@
   </si>
   <si>
     <t>Use this property to establish another catalogue in this catalogue.
-Note that deeply nested structures should be avoided, and can currently not be displayed in the National Health Data Catalogue.</t>
-  </si>
-  <si>
-    <t>If applicable, add URI to dcat:Catalog that is part of this catalogue</t>
+Note that deeply nested structures should be avoided, and cannot currently be displayed in the National Health Data Catalogue.</t>
+  </si>
+  <si>
+    <t>If applicable, add the URI of the dcat:Catalog that is part of this catalogue.</t>
   </si>
   <si>
     <t>home page</t>
@@ -410,7 +410,7 @@
     <t>dct:publisher</t>
   </si>
   <si>
-    <t>The organisation or individual that is holder of the intellectual property rights of a dataset. For more details about the publisher, see the class Agent. Example: Radboudumc.</t>
+    <t>The organisation or individual that is the holder of the intellectual property rights of a dataset. For more details about the publisher, see the class Agent. Example: Radboudumc.</t>
   </si>
   <si>
     <t>Adapted from v1</t>
@@ -449,13 +449,13 @@
     <t>service</t>
   </si>
   <si>
-    <t>A service that is listed in the catalog.</t>
+    <t>A service that is listed in the catalogue.</t>
   </si>
   <si>
     <t>dcat:service</t>
   </si>
   <si>
-    <t>Some datasets may have real-time Data Services (e.g., Beacon API counting individuals). IT teams should define the relationship between the catalog and the Data Service via this property. While crucial for interoperability, this property is not relevant for end-users to collect.</t>
+    <t>Some datasets may have real-time Data Services (e.g., Beacon API counting individuals). IT teams should define the relationship between the catalogue and the Data Service via this property. While crucial for interoperability, this property is not relevant for end users to collect.</t>
   </si>
   <si>
     <t>dcat:DataService</t>
@@ -488,7 +488,7 @@
     <t>dcat:themeTaxonomy</t>
   </si>
   <si>
-    <t>This property refers to a knowledge organisation system used to classify the Catalogue's Datasets. It must have at least the value NAL:data-theme as this is the mandatory controlled vocabulary for dcat:theme.</t>
+    <t>This property refers to a knowledge organisation system used to classify the Catalogue's Datasets. It must include at least the value NAL:data-theme as this is the mandatory controlled vocabulary for dcat:theme.</t>
   </si>
   <si>
     <t>skos:ConceptScheme</t>
@@ -503,7 +503,7 @@
     <t>dct:title</t>
   </si>
   <si>
-    <t>Provide a unique title for your catalog, which can be repeated in multiple languages. Example: Healthy Brain Study.</t>
+    <t>Provide a unique title for your catalogue, which can be repeated in multiple languages. Example: Healthy Brain Study.</t>
   </si>
   <si>
     <t>custom:purpose</t>
@@ -515,10 +515,10 @@
     <t>custom:retention_period</t>
   </si>
   <si>
-    <t>(issue on github)</t>
-  </si>
-  <si>
-    <t>issue on ckan github</t>
+    <t>(issue on GitHub)</t>
+  </si>
+  <si>
+    <t>issue on CKAN GitHub</t>
   </si>
   <si>
     <t>custom:status</t>
@@ -588,7 +588,7 @@
     <t>custom:analytics</t>
   </si>
   <si>
-    <t>If available, add URI to analytics distribution here</t>
+    <t>If available, add the URI for the analytics distribution here.</t>
   </si>
   <si>
     <t>code values</t>
@@ -609,7 +609,7 @@
     <t>coding system</t>
   </si>
   <si>
-    <t>Coding systems in use (ex: ICD-10-CM, DGRs, SNOMED=CT, ...)</t>
+    <t>Coding systems in use (e.g. ICD-10-CM, DGRs, SNOMED CT, ...)</t>
   </si>
   <si>
     <t>healthdcatap:hasCodingSystem</t>
@@ -636,15 +636,15 @@
     <t>custom:contact_</t>
   </si>
   <si>
-    <t>The creator (of the dataset) is the entity responsible for making the resource. According to Dutch databank and copyright law, this is in most cases the organisation / employer bearing investment risk, instead of an individual (e.g. individual researcher). Therefore, in many cases, this might be the same Agent as the dct:publisher, being the organisation (not a department or subdivision of the organisation) where the dataset was created.
-In case there are multiple (collaborating) organisations involved in data creation, all of them can be stated as dct:creator, as the model allows more than one creator.
+    <t>The creator (of the dataset) is the entity responsible for making the resource. According to Dutch databank and copyright law, this is in most cases the organisation/employer bearing investment risk, instead of an individual (e.g. an individual researcher). Therefore, in many cases, this might be the same Agent as the dct:publisher: the organisation (not a department or subdivision of the organisation) where the dataset was created.
+If there are multiple (collaborating) organisations involved in data creation, all of them can be stated as dct:creator, as the model allows more than one creator.
 In case you wish to credit other contributors to the dataset, you can use the prov:qualifiedAttribution property. This could be useful if you wish to indicate, for example, the funding organisation(s), collaborating organisation(s) or name specific individuals (e.g., principal investigator) involved in creating or managing the dataset.</t>
   </si>
   <si>
     <t>custom:creator_</t>
   </si>
   <si>
-    <t>Brief description of the dataset. You can repeat this property in multiple languages. Example: ''Collection of physiological data of Healthy Brain Study participants. This collection includes measurements via biowearables for heart rate, oxygenation, systolic and diastolic measures and stress levels.''</t>
+    <t>Brief description of the dataset. You can repeat this property in multiple languages. Example: ‘Collection of physiological data of Healthy Brain Study participants. This collection includes measurements via biowearables for heart rate, oxygenation, systolic and diastolic measures and stress levels.’</t>
   </si>
   <si>
     <t>distribution</t>
@@ -659,7 +659,7 @@
     <t>Metadata element used as a key link to the class Distribution.</t>
   </si>
   <si>
-    <t>fill in URI to dcat:Distribution</t>
+    <t>Enter the URI for dcat:Distribution.</t>
   </si>
   <si>
     <t>documentation</t>
@@ -671,7 +671,7 @@
     <t>foaf:page</t>
   </si>
   <si>
-    <t>The value of this property is the IRI directing to the web-page or document about the dataset.</t>
+    <t>The value of this property is the IRI pointing to the web page or document about the dataset.</t>
   </si>
   <si>
     <t>custom:documentation</t>
@@ -696,7 +696,7 @@
     <t>custom:frequency</t>
   </si>
   <si>
-    <t>The EU Vocabularies Name Authority Lists must be used for continents, countries and places that are in those lists; if a particular location is not in one of the mentioned Named Authority Lists, Geonames URIs must be used. For districts or neighbourhoods in NL, the Dutch vocab can be used. However, it might in many cases be desirable to keep the geographical coverage broader (e.g. indicating that NL is covered), to avoid exposing detailed information about subjects' locations.</t>
+    <t>The EU Vocabularies Named Authority Lists must be used for continents, countries and places that are in those lists; if a particular location is not in one of the mentioned Named Authority Lists, GeoNames URIs must be used. For districts or neighbourhoods in NL, the Dutch vocabulary can be used. However, it might in many cases be desirable to keep the geographical coverage broader (e.g. indicating that NL is covered), to avoid exposing detailed information about subjects' locations.</t>
   </si>
   <si>
     <t>has version</t>
@@ -708,7 +708,7 @@
     <t>dcat:hasVersion</t>
   </si>
   <si>
-    <t>Indicate the dataset which is the other version of the current dataset.</t>
+    <t>Indicate the dataset that is another version of the current dataset.</t>
   </si>
   <si>
     <t>custom:has_version</t>
@@ -739,7 +739,7 @@
   </si>
   <si>
     <t>Current status: Health-RI is currently working on a strategy for persistent identifiers for, among other things, datasets. Until a solid solution has been found, we propose the following temporary solution:
-If your data is published in a repository, fill in with the provided DOI (Example: https://doi.org/10.34894/ZLOYOJ). If not, use the identifier of the dataset as generated in the FAIR data point (FDP). Ensure that metadata is updated if your situation changes.</t>
+If your data is published in a repository, enter the provided DOI (Example: https://doi.org/10.34894/ZLOYOJ). If not, use the identifier of the dataset as generated in the FAIR data point (FDP). Ensure that metadata is updated if your situation changes.</t>
   </si>
   <si>
     <t>custom:alternate_identifier</t>
@@ -754,13 +754,13 @@
     <t>dcat:inSeries</t>
   </si>
   <si>
-    <t xml:space="preserve">This property points to which Dataset Series the Dataset is part of. </t>
+    <t xml:space="preserve">This property points to the Dataset Series of which the Dataset is part. </t>
   </si>
   <si>
     <t>dcat:DatasetSeries</t>
   </si>
   <si>
-    <t>If applicable, add URI to dataset series here</t>
+    <t>If applicable, add the URI for the dataset series here.</t>
   </si>
   <si>
     <t>is referenced by</t>
@@ -772,7 +772,7 @@
     <t>dct:isReferencedBy</t>
   </si>
   <si>
-    <t>The value of this property is the IRI of the doi to the publication or other related resource.
+    <t>The value of this property is the IRI of the DOI for the publication or other related resource.
 For example: https://doi.org/10.1186/s13690-021-00709-x</t>
   </si>
   <si>
@@ -884,7 +884,7 @@
     <t>adms:identifier</t>
   </si>
   <si>
-    <t>Examples for secondary identifiers are MAST/ADS, DataCite, DOI, EZID or W3ID (if not used for the original identifier). This property makes use of another, small class: adms:Identifier, where you provide the identifier and the name of the identifier schema (eg. DOI).</t>
+    <t>Examples of secondary identifiers include MAST/ADS, DataCite, DOI, EZID or W3ID (if not used for the original identifier). This property makes use of another small class: adms:Identifier, where you provide the identifier and the name of the identifier schema (e.g. DOI).</t>
   </si>
   <si>
     <t>adms:Identifier</t>
@@ -905,7 +905,7 @@
     <t>https://w3c.github.io/dpv/2.0/pd/</t>
   </si>
   <si>
-    <t>The different types of personal information that are collected in the dataset can be indicated with this property. Values can be picked from the dpv taxonomy (see controlled vocabulary column).
+    <t>The different types of personal information that are collected in the dataset can be indicated with this property. Values can be picked from the DPV taxonomy (see the Controlled vocabulary column).
 For example: dpv-pd:Gender</t>
   </si>
   <si>
@@ -921,13 +921,13 @@
     <t>healthdcatap:populationCoverage</t>
   </si>
   <si>
-    <t>This field is a free text description of the population covered in the dataset. For example, "Adults aged 18–65 diagnosed with type 2 diabetes in the Netherlands between 2015 and 2020".</t>
+    <t>This field is a free-text description of the population covered in the dataset. For example, "Adults aged 18–65 diagnosed with type 2 diabetes in the Netherlands between 2015 and 2020".</t>
   </si>
   <si>
     <t>custom:populatiion_coverage</t>
   </si>
   <si>
-    <t>This property identifies the organisation or individual responsible for making the dataset available. For datasets, this is typically the employer of the data creators. In simple cases, the dataset publisher may be the same as the catalog publisher. In more complex settings, such as when datasets come from multiple institutions within a consortium, the consortium should be listed as the publisher where possible. If no formal consortium can be specified, provide the information of the contributing organizations or individuals under dct:creator instead. For more details, refer to the Agent class.</t>
+    <t>This property identifies the organisation or individual responsible for making the dataset available. For datasets, this is typically the employer of the data creators. In simple cases, the dataset publisher may be the same as the catalogue publisher. In more complex settings, such as when datasets come from multiple institutions within a consortium, the consortium should be listed as the publisher where possible. If no formal consortium can be specified, provide information about the contributing organisations or individuals under dct:creator instead. For more details, refer to the Agent class.</t>
   </si>
   <si>
     <t>purpose</t>
@@ -1007,7 +1007,7 @@
     <t>prov:Attribution</t>
   </si>
   <si>
-    <t>fill in in 'Attribution' tab</t>
+    <t>Enter the value on the 'Attribution' tab.</t>
   </si>
   <si>
     <t>qualified relation</t>
@@ -1025,7 +1025,7 @@
     <t>dcat:Relationship</t>
   </si>
   <si>
-    <t>fill in in 'Relationship' tab</t>
+    <t>Enter the value on the 'Relationship' tab.</t>
   </si>
   <si>
     <t>quality annotation</t>
@@ -1043,7 +1043,7 @@
     <t>dqv:QualityCertificate</t>
   </si>
   <si>
-    <t>fill in in 'QualityCertificate' tab</t>
+    <t>Enter the value on the 'QualityCertificate' tab.</t>
   </si>
   <si>
     <r>
@@ -1098,13 +1098,13 @@
     <t>retention period</t>
   </si>
   <si>
-    <t>A temporal period which the dataset is available for secondary use.</t>
+    <t>A temporal period during which the dataset is available for secondary use.</t>
   </si>
   <si>
     <t>healthdcatap:retentionPeriod</t>
   </si>
   <si>
-    <t>fill in in 'Period of Time' tab</t>
+    <t>Enter the value on the 'PeriodOfTime' tab.</t>
   </si>
   <si>
     <t>sample</t>
@@ -1116,10 +1116,10 @@
     <t>adms:sample</t>
   </si>
   <si>
-    <t>This property makes use of the dcat:Distribution class to describe a sample distribution of the dataset, which can be anonymized or synthetic data, or the data dictionary provided in CSVW format. This is currently further developed by the TEHDAS2 program. More information can be found here: https://healthdcat-ap.github.io/#sample-distribution</t>
-  </si>
-  <si>
-    <t>If available, add URI to sample distribution here</t>
+    <t>This property makes use of the dcat:Distribution class to describe a sample distribution of the dataset, which can consist of anonymised or synthetic data, or a data dictionary provided in CSVW format. This is currently being further developed by the TEHDAS2 programme. More information can be found here: https://healthdcat-ap.github.io/#sample-distribution</t>
+  </si>
+  <si>
+    <t>If available, add the URI for the sample distribution here.</t>
   </si>
   <si>
     <t>source</t>
@@ -1134,7 +1134,7 @@
     <t>Indicate the dataset on which this described dataset is based.</t>
   </si>
   <si>
-    <t>If applicable, add URI to source dataset here</t>
+    <t>If applicable, add the URI for the source dataset here.</t>
   </si>
   <si>
     <t>status</t>
@@ -1165,7 +1165,7 @@
     <t>dcat:temporalResolution</t>
   </si>
   <si>
-    <t>If the dataset is a time-series, this should correspond to the spacing of items in the series. For other kinds of dataset, this property will usually indicate the smallest time difference between items in the dataset. The time period has to be provided in the xsd:duration format.</t>
+    <t>If the dataset is a time-series, this should correspond to the spacing of items in the series. For other kinds of datasets, this property will usually indicate the smallest time difference between items in the dataset. The time period has to be provided in the xsd:duration format.</t>
   </si>
   <si>
     <t>xsd:duration</t>
@@ -1219,7 +1219,7 @@
     <t>adms:versionNotes</t>
   </si>
   <si>
-    <t>Provide a short description of changes made to the dataset from the previous version.</t>
+    <t>Provide a short description of changes made to the dataset since the previous version.</t>
   </si>
   <si>
     <t>was generated by</t>
@@ -1284,7 +1284,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> of additional classes  (additional instances of Dataset, DatasetSeries, DataService or Catalogue)</t>
+      <t xml:space="preserve"> of additional classes (additional instances of Dataset, DatasetSeries, DataService or Catalogue).</t>
     </r>
   </si>
   <si>
@@ -1313,7 +1313,7 @@
 Wikidata: https://www.wikidata.org/wiki/Wikidata:Main_Page</t>
   </si>
   <si>
-    <t>Specify the entity (person or organization) by providing an identifier. We recommend using an ORCID identifier for a person or ROR identifier for an organization. Dutch government organizations are listed in TOOI. If these are not available, you can use ISNI, or Wikidata or any other identifier you may have. If you have multiple identifiers, you should provide them all.</t>
+    <t>Specify the entity (person or organisation) by providing an identifier. We recommend using an ORCID identifier for a person or a ROR identifier for an organisation. Dutch government organisations are listed in TOOI. If these are not available, you can use ISNI, Wikidata or any other identifier you may have. If you have multiple identifiers, you should provide them all.</t>
   </si>
   <si>
     <t>HRI v1</t>
@@ -1331,7 +1331,7 @@
     <t>foaf:name</t>
   </si>
   <si>
-    <t>This property refers to the given name of the entity. Example: Jane Doe (for a person) and Radboudumc (for an organization). This property can be repeated for different versions of the name (e.g. the name in different languages).</t>
+    <t>This property refers to the given name of the entity. Example: Jane Doe (for a person) and Radboudumc (for an organisation). This property can be repeated for different versions of the name (e.g. the name in different languages).</t>
   </si>
   <si>
     <t>_name</t>
@@ -1340,7 +1340,7 @@
     <t>publisher note</t>
   </si>
   <si>
-    <t>A description of the publisher activities.</t>
+    <t>A description of the publisher's activities.</t>
   </si>
   <si>
     <t>healthdcatap:publishernote</t>
@@ -1358,7 +1358,7 @@
     <t>https://raw.githubusercontent.com/SEMICeu/ADMS-AP/master/purl.org/ADMS_SKOS_v1.00.rdf</t>
   </si>
   <si>
-    <t>This property should be filled using ADMS vocabulary (http://purl.org/adms/publishertype/1.0)</t>
+    <t>This property should be filled using ADMS vocabulary (http://purl.org/adms/publishertype/1.0).</t>
   </si>
   <si>
     <t>_type</t>
@@ -1411,7 +1411,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> of additional classes ( (additional instances of Dataset, DatasetSeries, DataService or Catalogue)</t>
+      <t xml:space="preserve"> of additional classes (additional instances of Dataset, DatasetSeries, DataService or Catalogue).</t>
     </r>
   </si>
   <si>
@@ -1481,10 +1481,10 @@
     <t>resource:access_services</t>
   </si>
   <si>
-    <t>If applicable, fill in URI to dcat:DatasService</t>
-  </si>
-  <si>
-    <t>access url</t>
+    <t>If applicable, enter the URI for dcat:DataService.</t>
+  </si>
+  <si>
+    <t>access URL</t>
   </si>
   <si>
     <t>A URL of the resource that gives access to a distribution of the dataset. E.g., landing page, feed, SPARQL endpoint.</t>
@@ -1529,7 +1529,7 @@
     <t>spdx:checksum</t>
   </si>
   <si>
-    <t>The checksum is related to the downloadURL. This property makes use of the spdx:Checksum class, which itself has two properties to indicate checksum algorithm and checksum value (see Checksum class for further details).</t>
+    <t>The checksum is related to the downloadURL. This property makes use of the spdx:Checksum class, which itself has two properties to indicate the checksum algorithm and checksum value (see Checksum class for further details).</t>
   </si>
   <si>
     <t>spdx:Checksum</t>
@@ -1538,13 +1538,13 @@
     <t>resource:hash_algorithm/resource:hash_algorithm</t>
   </si>
   <si>
-    <t>fill in in 'Checksum' tab</t>
+    <t>Enter the value on the 'Checksum' tab.</t>
   </si>
   <si>
     <t>compression format</t>
   </si>
   <si>
-    <t>The compression format of the distribution in which the data is contained in a compressed form, e.g., to reduce the size of the downloadable file.</t>
+    <t>The compression format of the distribution in which the data is compressed, e.g., to reduce the size of the downloadable file.</t>
   </si>
   <si>
     <t>dcat:compressFormat</t>
@@ -1608,7 +1608,7 @@
   </si>
   <si>
     <r>
-      <t>Indicates the </t>
+      <t xml:space="preserve">Indicates the </t>
     </r>
     <r>
       <rPr>
@@ -1627,7 +1627,7 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t xml:space="preserve"> used in the Distribution, indicated with a value from the EU controlled vocabulary. Not all distributions might have a language, for example imaging data.
+      <t xml:space="preserve"> used in the Distribution, using a value from the EU controlled vocabulary. Not all distributions might have a language, for example imaging data.
 Note that here the Health-RI model diverges from DCAT-AP NL, which allows a maximum of 1 language per Distribution. The Health-RI model allows multiple languages in the same Distribution.</t>
     </r>
   </si>
@@ -1635,10 +1635,10 @@
     <t>resource:language</t>
   </si>
   <si>
-    <t>license</t>
-  </si>
-  <si>
-    <t>For public data, use a Creative Commons (CC) license (see Geonovum options in the Controlled Vocabulary column). For most National Health Data Catalogue distributions, where data is not public, use the 'not open' license from Geonovum and specify data reuse agreements in the dct:rights property.</t>
+    <t>licence</t>
+  </si>
+  <si>
+    <t>For public data, use a Creative Commons (CC) licence (see Geonovum options in the Controlled Vocabulary column). For most National Health Data Catalogue distributions, where data is not public, use the 'not open' licence from Geonovum and specify data reuse agreements in the dct:rights property.</t>
   </si>
   <si>
     <t>resource:license</t>
@@ -1662,7 +1662,7 @@
     <t>dcat:mediaType</t>
   </si>
   <si>
-    <t>Use the specified vocabularies, prioritizing IANA media types whenever possible. If unavailable, consider other ontologies, such as ZonMw generic terms, to describe the format.
+    <t>Use the specified vocabularies, prioritising IANA media types whenever possible. If unavailable, consider other ontologies, such as ZonMw generic terms, to describe the format.
 Example: https://www.iana.org/assignments/media-types/text/csv (for csv)
 If IANA media types do not sufficiently describe the format, use "format" to describe it in more detail.</t>
   </si>
@@ -1697,7 +1697,7 @@
     <t>healthdcatap:retentionperiod</t>
   </si>
   <si>
-    <t>fill in in 'Periof of Time' tab</t>
+    <t>Enter the value on the 'PeriodOfTime' tab.</t>
   </si>
   <si>
     <t>resource:rights</t>
@@ -1707,16 +1707,16 @@
 EU Vocabularies Distribution Status</t>
   </si>
   <si>
-    <t>It MUST take one of the values Completed, Deprecated, Under Development, Withdrawn from the provided controlled vocabulary.</t>
+    <t>It MUST take one of the following values from the provided controlled vocabulary: Completed, Deprecated, Under Development or Withdrawn.</t>
   </si>
   <si>
     <t>resource:status</t>
   </si>
   <si>
-    <t>If applicable, this property indicates the minimum time period resolvable in the dataset distribution, expressed in xsd:duration format (see for more information here: https://www.w3schools.com/xml/schema_dtypes_date.asp)</t>
-  </si>
-  <si>
-    <t>A title given to the distribution. e.g., Data Access Request of Healthy Brain study</t>
+    <t>If applicable, this property indicates the minimum time period resolvable in the dataset distribution, expressed in xsd:duration format (for more information, see: https://www.w3schools.com/xml/schema_dtypes_date.asp).</t>
+  </si>
+  <si>
+    <t>A title given to the distribution, e.g. Data Access Request for the Healthy Brain Study</t>
   </si>
   <si>
     <t>resource:name</t>
@@ -1734,7 +1734,7 @@
     <t>data_series::contact</t>
   </si>
   <si>
-    <t xml:space="preserve">Briefly describe the dataset series in the catalog. You can repeat this in multiple languages. </t>
+    <t xml:space="preserve">Briefly describe the dataset series in the catalogue. You can repeat this in multiple languages. </t>
   </si>
   <si>
     <t>data_series::modified</t>
@@ -1749,7 +1749,7 @@
     <t>This is not equal to the most recently modified dataset in the collection of the dataset series.</t>
   </si>
   <si>
-    <t xml:space="preserve">The publisher of the dataset series may not be the publisher of all datasets.  E.g. a digital archive could take over the publishing of older datasets in the series. </t>
+    <t xml:space="preserve">The publisher of the dataset series may not be the publisher of all datasets. For example, a digital archive could take over the publishing of older datasets in the series. </t>
   </si>
   <si>
     <t>data_series::publisher</t>
@@ -1761,7 +1761,7 @@
     <t>data_series:issued</t>
   </si>
   <si>
-    <t>When temporal coverage is a dimension in the dataset series then the temporal coverage of each dataset in the collection should be part of the temporal coverage. In that case, an open-ended value is recommended, e.g. after 2012.</t>
+    <t>When temporal coverage is a dimension in the dataset series, the temporal coverage of each dataset in the collection should be part of the series' temporal coverage. In that case, an open-ended value is recommended, e.g. after 2012.</t>
   </si>
   <si>
     <t>data_series::temporal</t>
@@ -1774,7 +1774,7 @@
   </si>
   <si>
     <r>
-      <t>Information that indicates whether the Dataset is publicly accessible, has access restrictions or is not public. This property is required to adopt one of the predefined values listed in the </t>
+      <t>Information that indicates whether the Dataset is publicly accessible, has access restrictions or is not public. This property must take one of the predefined values listed in the </t>
     </r>
     <r>
       <rPr>
@@ -1831,10 +1831,10 @@
     <t>access_service:description</t>
   </si>
   <si>
-    <t>end point description</t>
-  </si>
-  <si>
-    <t>A description of the services available via the end-points, including their operations, parameters etc.</t>
+    <t>endpoint description</t>
+  </si>
+  <si>
+    <t>A description of the services available via the endpoints, including their operations, parameters, etc.</t>
   </si>
   <si>
     <t>dcat:endpointDescription</t>
@@ -1846,7 +1846,7 @@
     <t>access_service:endpoint_description</t>
   </si>
   <si>
-    <t>end point URL</t>
+    <t>endpoint URL</t>
   </si>
   <si>
     <t>The root location or primary endpoint of the service (a Web-resolvable IRI).</t>
@@ -1870,22 +1870,22 @@
     <t>Provide a unique identifier for the data service. This could be a globally unique and persistent identifier, such as a DOI, URN, or UUID. If no persistent identifier is available, you may use the accessURL or endpointURL as the identifier, provided it is stable and unique to the service.</t>
   </si>
   <si>
-    <t>landing Page</t>
-  </si>
-  <si>
-    <t>A Web page that can be navigated to in a Web browser to gain access to the catalog, a dataset, its distributions and/or additional information.</t>
+    <t>landing page</t>
+  </si>
+  <si>
+    <t>A Web page that can be navigated to in a Web browser to gain access to the catalogue, a dataset, its distributions and/or additional information.</t>
   </si>
   <si>
     <t>dcat:landingPage</t>
   </si>
   <si>
-    <t>It is intended to point to a landing page at the original data service provider, not to a page on a site of a third party, such as an aggregator.</t>
+    <t>It is intended to point to a landing page at the original data service provider, not to a page on a third-party site, such as an aggregator.</t>
   </si>
   <si>
     <t>Indicates the natural language used in the data service, indicated with a value from the EU controlled vocabulary.</t>
   </si>
   <si>
-    <t>For public data, use a Creative Commons (CC) license (see Geonovum options in the Controlled Vocabulary column). For most National Health Data Catalogue data services, where data is not public, use the 'not open' license from Geonovum and specify data reuse agreements in the dct:rights property.</t>
+    <t>For public data, use a Creative Commons (CC) licence (see Geonovum options in the Controlled Vocabulary column). For most National Health Data Catalogue data services, where data is not public, use the 'not open' licence from Geonovum and specify data reuse agreements in the dct:rights property.</t>
   </si>
   <si>
     <t>access_service:license</t>
@@ -1894,10 +1894,10 @@
     <t>This property indicates the date of the last changes to the dataset, not the metadata record. An absent value may mean the resource hasn't changed since publication, the modification date is unknown, or the resource is continuously updated.</t>
   </si>
   <si>
-    <t>fill in in 'adms_Identifier' tab</t>
-  </si>
-  <si>
-    <t>The organization or individual responsible for making the data service available. In the context of data services, the publisher is typically the organization that manages or provides access to the service. For details, see the class Agent.</t>
+    <t>Enter the value on the 'adms_Identifier' tab.</t>
+  </si>
+  <si>
+    <t>The organisation or individual responsible for making the data service available. In the context of data services, the publisher is typically the organisation that manages or provides access to the service. For details, see the class Agent.</t>
   </si>
   <si>
     <t>serves dataset</t>
@@ -1915,13 +1915,13 @@
     <t>access_service:serves_dataset</t>
   </si>
   <si>
-    <t>fill in URI to dcat:Dataset that this data service serves</t>
+    <t>Enter the URI for the dcat:Dataset that this data service serves.</t>
   </si>
   <si>
     <t>This property should use a controlled vocabulary. In the Health Data Catalogue, most data services will use NAL:data-theme 'HEAL', but additional values from the same vocabulary are allowed.</t>
   </si>
   <si>
-    <t>Provide a unique title for your data service, which can be repeated in multiple languages. Example: Patient counts per available diagnosis</t>
+    <t>Provide a unique title for your data service, which can be repeated in multiple languages. Example: Patient counts per available diagnosis.</t>
   </si>
   <si>
     <t>access_service:title</t>
@@ -1959,7 +1959,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> of additional classes (additional instances of Dataset or DataService)</t>
+      <t xml:space="preserve"> of additional classes (additional instances of Dataset or DataService).</t>
     </r>
   </si>
   <si>
@@ -2045,7 +2045,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> of additional classes (additional instances of Catalogue, Dataset, Distribution or Dataset Series)</t>
+      <t xml:space="preserve"> of additional classes (additional instances of Catalogue, Dataset, Distribution or Dataset Series).</t>
     </r>
   </si>
   <si>
@@ -2067,13 +2067,13 @@
     <t>dcat:startDate</t>
   </si>
   <si>
-    <t>Value: qualified Attribution (Dataset A)</t>
-  </si>
-  <si>
-    <t>Value: qualified Attribution (Dataset B)</t>
-  </si>
-  <si>
-    <t>Value: qualified Attribution (Dataset C)</t>
+    <t>Value: qualified attribution (Dataset A)</t>
+  </si>
+  <si>
+    <t>Value: qualified attribution (Dataset B)</t>
+  </si>
+  <si>
+    <t>Value: qualified attribution (Dataset C)</t>
   </si>
   <si>
     <r>
@@ -2099,14 +2099,14 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> of additional classes (additional instances of Dataset)</t>
+      <t xml:space="preserve"> of additional classes (additional instances of Dataset).</t>
     </r>
   </si>
   <si>
     <t>agent</t>
   </si>
   <si>
-    <t>The prov:agent property references a prov:Agent which influenced a resource.</t>
+    <t>The prov:agent property references a prov:Agent that influenced a resource.</t>
   </si>
   <si>
     <t>prov:agent</t>
@@ -2131,16 +2131,16 @@
   <si>
     <t>Choose one of the roles as listed in the controlled vocabulary. Note that for HealthDCAT-AP, the list of roles might be extended in the future.
 Example: https://standards.iso.org/iso/19115/resources/Codelists/gml/CI_RoleCode.xml#processor
-Next to the CI_RoleCode, we also propose to use the CRediT Taxonomy to specify roles of contributors.</t>
-  </si>
-  <si>
-    <t>Value qualified Relation (Dataset A)</t>
-  </si>
-  <si>
-    <t>Value qualified Relation (Dataset B)</t>
-  </si>
-  <si>
-    <t>Value qualified Relation (Dataset C)</t>
+In addition to CI_RoleCode, we also propose to use the CRediT Taxonomy to specify roles of contributors.</t>
+  </si>
+  <si>
+    <t>Value: qualified relation (Dataset A)</t>
+  </si>
+  <si>
+    <t>Value: qualified relation (Dataset B)</t>
+  </si>
+  <si>
+    <t>Value: qualified relation (Dataset C)</t>
   </si>
   <si>
     <r>
@@ -2166,7 +2166,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t>of additional classes (additional instances of Dataset)</t>
+      <t>of additional classes (additional instances of Dataset).</t>
     </r>
   </si>
   <si>
@@ -2226,7 +2226,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> of additional classes (additional instances of Dataset)</t>
+      <t xml:space="preserve"> of additional classes (additional instances of Dataset).</t>
     </r>
   </si>
   <si>
@@ -2240,7 +2240,7 @@
   </si>
   <si>
     <t>This property has to be filled with the same value as the dct:identifier of the dataset described, in order to link the quality certificate to that dataset.
-See also example in HealthDCAT-AP: https://healthdcat-ap.github.io/#dqvhasqualityannotation</t>
+See also the example in HealthDCAT-AP: https://healthdcat-ap.github.io/#dqvhasqualityannotation</t>
   </si>
   <si>
     <t>body</t>
@@ -2345,7 +2345,7 @@
     <t xml:space="preserve">foaf:primaryTopic </t>
   </si>
   <si>
-    <t xml:space="preserve">A catalogue record will refer to one entity in a catalogue. This can be either a Dataset or a Data Service. To ensure an unambigous reading of the cardinality the range is set to Catalogued Resource. However it is not the intend with this range to require the explicit use of the class Catalogued Record. As abstract class, an subclass should be used. </t>
+    <t xml:space="preserve">A catalogue record will refer to one entity in a catalogue. This can be either a Dataset or a Data Service. To ensure an unambiguous reading of the cardinality, the range is set to Catalogued Resource. However, this range is not intended to require the explicit use of the class Catalogued Record. Since this is an abstract class, a subclass should be used. </t>
   </si>
   <si>
     <t xml:space="preserve">dcat:Resource </t>
@@ -2404,7 +2404,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> of additional classes (additional instances of Distribution)</t>
+      <t xml:space="preserve"> of additional classes (additional instances of Distribution).</t>
     </r>
   </si>
   <si>
@@ -2420,7 +2420,7 @@
     <t>https://spdx.org/rdf/terms/#d4e2129</t>
   </si>
   <si>
-    <t>Choose one member of the checksum algorithm members as indicated on the webpage linked in the Controlled Vocabulary column.</t>
+    <t>Choose one of the checksum algorithms as indicated on the webpage linked in the Controlled Vocabulary column.</t>
   </si>
   <si>
     <t>spdx:ChecksumAlgorithm (IRI)</t>
@@ -2440,13 +2440,13 @@
   <si>
     <t>It is preferred to provide a general email address of the appropriate institution or department instead of a personal email address, even if an individual is described with this instance of foaf:Agent.
 This protects their privacy and enables contact about the resource even after the individual has left the institution.
-The email address has to be provided starting with mailto: prefix.
+The email address must start with the mailto: prefix.
 For example: mailto:info@example.com</t>
   </si>
   <si>
     <t>It is preferred to provide a general email address of the appropriate institution or department instead of a personal email address, even if an individual is described with this instance of vcard:Kind.
 This protects their privacy and enables contact about the resource even after the individual has left the institution.
-The email address has to be provided starting with mailto: prefix.
+The email address must start with the mailto: prefix.
 For example: mailto:info@example.com</t>
   </si>
   <si>
@@ -2459,21 +2459,21 @@
   <si>
     <t>The ELI of the EHDS was published in March 2025 and can now be included as the applicable legislation mandating that the dataset has to be made public.
 For health datasets, the value must include the ELI of the EHDS Regulation (http://data.europa.eu/eli/reg/2025/327/oj).
-As multiple legislations may apply to the resource the maximum cardinality is not limited. Note that the relation with other legislations is complex and is being looked into by legal experts.
-While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property (also in Datasets) described the legal basis for initial collection and processing of (personal) data.</t>
-  </si>
-  <si>
-    <t>The legal basis can be provided as a value from the dpv taxonomy (see Controlled vocabulary column).
+As multiple pieces of legislation may apply to the resource, the maximum cardinality is not limited. Note that the relationship with other legislation is complex and is being looked into by legal experts.
+While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property (also in Datasets) describes the legal basis for initial collection and processing of (personal) data.</t>
+  </si>
+  <si>
+    <t>The legal basis can be provided as a value from the DPV taxonomy (see the Controlled vocabulary column).
 While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property describes the legal basis for initial collection and processing of (personal) data.
 This property should always be filled if the dataset contains personal data and the applicable legislation is GDPR.
-Example value for this property could be: dpv:Consent</t>
-  </si>
-  <si>
-    <t>One (or many) categories or sub-categories of the purposes can be chosen from the taxonomy provided by dpv (see controlled vocabulary column). Try to be as specific as possible.
-Example value could be: dpv:ResearchAndDevelopment.</t>
-  </si>
-  <si>
-    <t>Indicate with this property in case the Dataset is only available for secondary use for a specific period of time (e.g. due to data protection, contractual, or project constraints).
+An example value for this property could be dpv:Consent.</t>
+  </si>
+  <si>
+    <t>One or more categories or sub-categories of purposes can be chosen from the taxonomy provided by dpv (see the Controlled vocabulary column). Try to be as specific as possible.
+An example value could be dpv:ResearchAndDevelopment.</t>
+  </si>
+  <si>
+    <t>Use this property if the Dataset is only available for secondary use for a specific period of time (e.g. due to data protection, contractual, or project constraints).
 This property makes use of the class dct:PeriodOfTime, in which a start and end date can be provided.
 If the Dataset is available indefinitely, leave the property empty (cardinality is 0..1; it is only meaningful when a retention limit applies).
 If only a start is known, provide dcat:startDate only (open-ended interval, as allowed by dct:PeriodOfTime).
@@ -2576,7 +2576,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Display"/>
       </rPr>
-      <t>: The variables  have been added to the metadata model version 2.1 for testing purposes. For now it is not yet planned to be added to the national catalogue's front end.
+      <t>: The variables have been added to the metadata model version 2.1 for testing purposes. For now, their inclusion in the national catalogue's front end is not yet planned.
 Use this property to link a structured dataset to a CSVW TableGroup that documents its data variables, columns, or fields in a machine-readable way.</t>
     </r>
   </si>
@@ -2602,16 +2602,16 @@
     <t>Value: table 2</t>
   </si>
   <si>
-    <t>Add more columns if you need to describe additional instances of csvw:TableGroup</t>
+    <t>Add more columns if you need to describe additional instances of csvw:TableGroup.</t>
   </si>
   <si>
     <t>csvw:TableGroup</t>
   </si>
   <si>
-    <t>fill in in 'TableGroup' tab</t>
-  </si>
-  <si>
-    <t>fill in in 'TableGroup'  tab</t>
+    <t>Enter the value on the 'TableGroup' tab.</t>
+  </si>
+  <si>
+    <t>Enter the value on the 'TableGroup' tab.</t>
   </si>
   <si>
     <t>url</t>
@@ -2626,7 +2626,7 @@
     <t>Table title.</t>
   </si>
   <si>
-    <t xml:space="preserve">A keyword or tag describing the table.	</t>
+    <t xml:space="preserve">A keyword or tag describing the table.</t>
   </si>
   <si>
     <t>A variable (column) defines metadata about one field in the CSV file.</t>
@@ -2641,7 +2641,7 @@
     <t>csvw:column</t>
   </si>
   <si>
-    <t>The URL should be a valid IRI and should point to the CSV file (synthetic, anonymized representation of the real data) for this table.</t>
+    <t>The URL should be a valid IRI and should point to the CSV file (a synthetic, anonymised representation of the real data) for this table.</t>
   </si>
   <si>
     <t>Used to provide a human-readable title for the table. Can appear in multiple languages.</t>
@@ -2656,7 +2656,7 @@
     <t>csvw:Column</t>
   </si>
   <si>
-    <t>Add more columns if you need to describe additional instances of csvw:Table</t>
+    <t>Add more columns if you need to describe additional instances of csvw:Table.</t>
   </si>
   <si>
     <t>datatype</t>
@@ -2699,7 +2699,7 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Should match the </t>
+      <t xml:space="preserve">The value should match the </t>
     </r>
     <r>
       <rPr>
@@ -2719,7 +2719,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> of one of the CSVW types as defined in the Built-in datatypes from XML Schema. https://w3c.github.io/csvw/metadata/#datatypes Example: string, integer, boolean …</t>
+      <t xml:space="preserve"> of one of the CSVW types as defined in the Built-in datatypes from XML Schema. See: https://w3c.github.io/csvw/metadata/#datatypes
+Example: string, integer, boolean …</t>
     </r>
   </si>
   <si>
@@ -3179,7 +3180,7 @@
     <t>availability</t>
   </si>
   <si>
-    <t>An indication how long it is planned to keep the Distribution of the Dataset available.</t>
+    <t>An indication of how long it is planned to keep the Distribution of the Dataset available.</t>
   </si>
   <si>
     <t>dcatap:availability</t>
@@ -3209,7 +3210,7 @@
         <scheme val="major"/>
       </rPr>
       <t>: This property will be deprecated in the upcoming major release. It is recommended to indicate the planned availability of the distribution with the newly added Distribution.availability property. 
-Indicate with this property in case the Distribution is only available for secondary use for a specific period of time (e.g. due to data protection, contractual, or project constraints).
+Use this property if the Distribution is only available for secondary use for a specific period of time (e.g. due to data protection, contractual, or project constraints).
 This property makes use of the class dct:PeriodOfTime, in which a start and end date can be provided.
 If the Distribution is available indefinitely, leave the property empty (cardinality is 0..1; it is only meaningful when a retention limit applies).
 If only a start is known, provide dcat:startDate only (open-ended interval, as allowed by dct:PeriodOfTime).
@@ -3265,7 +3266,7 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> for identifiers of the Dataset, such as DOI; use </t>
+      <t xml:space="preserve"> for identifiers of the Dataset, such as a DOI; use </t>
     </r>
     <r>
       <rPr>
@@ -3327,7 +3328,7 @@
     </r>
   </si>
   <si>
-    <t>Information about how the data was collected, including methodologies, tools, and protocols used. This property can be repeated for different versions of the provenance (e.g. the provenance in different languages).
+    <t>Information about how the data was collected, including methodologies, tools, and protocols used. This property can be repeated for different versions of the provenance (e.g. in different languages).
 This is where the collection-method statements not captured by dedicated properties can be listed.</t>
   </si>
   <si>
@@ -3341,7 +3342,7 @@
   </si>
   <si>
     <t>Use this property to indicate which anatomical parts of the body are covered by the Dataset. Select the relevant anatomical structure from SNOMED CT. Multiple anatomical locations can be provided.
-Example: Dataset containing lung imaging data can use Lung structure (http://snomed.info/id/39607008).</t>
+Example: A dataset containing lung imaging data can use Lung structure (http://snomed.info/id/39607008).</t>
   </si>
   <si>
     <t>domain of the data</t>
@@ -3382,8 +3383,8 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t>: The use of wikidata URIs will be replaced with the terms from a controlled vocabulary in the next major release.
-This property provides information on which coding systems are in use in your dataset. For this, wikidata URIs must be used.</t>
+      <t>: The use of Wikidata URIs will be replaced with the terms from a controlled vocabulary in the next major release.
+This property provides information on which coding systems are in use in your dataset. For this, Wikidata URIs must be used.</t>
     </r>
   </si>
   <si>
@@ -3404,8 +3405,8 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t>: The use of wikidata URIs will be replaced with the terms from a controlled vocabulary in the next major release.
-If your data conforms to an established standard or specification, use this property to indicate which one. The wikidata URI of the specification must be used. Example: https://www.wikidata.org/wiki/Q19597236 for FHIR.</t>
+      <t>: The use of Wikidata URIs will be replaced with the terms from a controlled vocabulary in the next major release.
+If your data conforms to an established standard or specification, use this property to indicate which one. The Wikidata URI of the specification must be used. Example: https://www.wikidata.org/wiki/Q19597236 for FHIR.</t>
     </r>
   </si>
   <si>
@@ -3424,8 +3425,8 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Display"/>
       </rPr>
-      <t>: The use of wikidata URIs will be replaced with the terms from a controlled vocabulary in the next major release.
-This property is a structured way to tag the dataset with different health themes. This could include, for example, the specific disease the dataset is about. More details can be provided, if desirable, in the keywords property.  The wikidata URI of the health theme must be used here.</t>
+      <t>: The use of Wikidata URIs will be replaced with the terms from a controlled vocabulary in the next major release.
+This property is a structured way to tag the dataset with different health themes. This could include, for example, the specific disease the dataset is about. More details can be provided, if desirable, in the keywords property.  The Wikidata URI of the health theme must be used here.</t>
     </r>
   </si>
   <si>
@@ -3466,7 +3467,7 @@
     </r>
   </si>
   <si>
-    <t>A statement that concerns all rights not addressed in fields License or Access rights. In case of not open data (as specified in the dct:licence property), further agreements regarding data reuse (e.g. Data Transfer Agreement, DTA) should be stated in this property.
+    <t>A statement that concerns all rights not addressed in the Licence or Access rights fields. For data that is not open (as specified in the dct:license property), further agreements regarding data reuse (e.g. Data Transfer Agreement, DTA) should be stated in this property.
 The rights statement should be a free-text statement placed at a web-accessible location such that the value of this property is the IRI pointing to that statement.</t>
   </si>
   <si>
@@ -3490,7 +3491,7 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> be used to provide the email address of the Agent, specified using fully qualified mailto: URI scheme RFC6068. The email </t>
+      <t xml:space="preserve"> be used to provide the email address of the Agent, specified using the fully qualified mailto: URI scheme defined in RFC 6068. The email </t>
     </r>
     <r>
       <rPr>
@@ -3542,8 +3543,8 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t>: The use of wikidata URIs will be replaced with free text in the next major release.
-Inside this property, you can provide the coding system of the dataset in the form of wikidata URI (example: https://www.wikidata.org/entity/P494 for ICD-10 ID) and the URI of the value that describes the dataset (example: https://icd.who.int/browse10/2019/en#/Y59.0 for viral vaccines)</t>
+      <t>: The use of Wikidata URIs will be replaced with free text in the next major release.
+Inside this property, you can provide the coding system of the dataset in the form of a Wikidata URI (example: https://www.wikidata.org/entity/P494 for ICD-10 ID) and the URI of the value that describes the dataset (example: https://icd.who.int/browse10/2019/en#/Y59.0 for viral vaccines).</t>
     </r>
   </si>
   <si>
@@ -3563,19 +3564,19 @@
     <t>rdfs:label</t>
   </si>
   <si>
-    <t>In this context the definition should be considered as: A textual statement describing the provenance of the Dataset, including information about its origin, history, or activities involved in its creation or modification.</t>
+    <t>In this context, the definition should be considered as: A textual statement describing the provenance of the Dataset, including information about its origin, history, or activities involved in its creation or modification.</t>
   </si>
   <si>
     <t>dct:ProvenanceStatement</t>
   </si>
   <si>
-    <t>Provide a short textual statement describing the provenance of the Dataset, such as its origin, how it was created or collected, or any relevant processing or transformations it has undergone. This statement should describe the provenance of the Dataset as a whole and be provided as free text.  You can repeat this property in multiple languages</t>
+    <t>Provide a short textual statement describing the provenance of the Dataset, such as its origin, how it was created or collected, or any relevant processing or transformations it has undergone. This statement should describe the provenance of the Dataset as a whole and be provided as free text. You can repeat this property in multiple languages.</t>
   </si>
   <si>
     <t>Value: activity (Dataset A)</t>
   </si>
   <si>
-    <t>Value:activity (Dataset B)</t>
+    <t>Value: activity (Dataset B)</t>
   </si>
   <si>
     <t>Value: activity (Dataset C)</t>
@@ -3590,7 +3591,7 @@
     <t>Value: provenance (Dataset 2)</t>
   </si>
   <si>
-    <t>Add more columns if you need to describe additional instances of dct:ProvenanceStatement for provenance of additional classes (additional instances of Dataset)</t>
+    <t>Add more columns if you need to describe additional instances of dct:ProvenanceStatement for provenance of additional classes (additional instances of Dataset).</t>
   </si>
   <si>
     <t>ProvenanceStatement</t>
@@ -3610,7 +3611,8 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Select data domain(s) from the predefined value list, available at this link: https://github.com/Health-RI/health-ri-metadata/blob/v2.1-changes/Formalisation(shacl)/Core/ValueLists/edam-has-topic.tsv </t>
+      <t xml:space="preserve">Select data domain(s) from the predefined value list, available at this link: https://github.com/Health-RI/health-ri-metadata/blob/v2.1-changes/Formalisation(shacl)/Core/ValueLists/edam-has-topic.tsv
+</t>
     </r>
     <r>
       <rPr>
@@ -3629,7 +3631,7 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t>: This is a temporary location and it will change with the release . 
+      <t>: This is a temporary location and it will change with the release. 
 A data domain refers to the broader scientific or health-related area covered by the Dataset. Select the domain that best represents the Dataset as a whole, rather than a specific data element within it. If the dataset contains data from more than one domain, you can select multiple.
 See the property "measurement technique" for more information about the technique(s) used to generate the data in the Dataset.</t>
     </r>
@@ -3673,8 +3675,9 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Select a suitable value or suitable values from the value list to indicate the technique(s) used to generate data in the dataset.
-The value list is  available at this link: https://github.com/Health-RI/health-ri-metadata/blob/v2.1-changes/Formalisation(shacl)/Core/ValueLists/schema-measurement-technique.tsv </t>
+      <t xml:space="preserve">Select one or more suitable values from the value list to indicate the technique(s) used to generate data in the dataset.
+The value list is available at this link: https://github.com/Health-RI/health-ri-metadata/blob/v2.1-changes/Formalisation(shacl)/Core/ValueLists/schema-measurement-technique.tsv
+</t>
     </r>
     <r>
       <rPr>
@@ -3693,14 +3696,14 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t xml:space="preserve">: This is a temporary location and it will change with the next release . </t>
+      <t xml:space="preserve">: This is a temporary location and it will change with the next release. </t>
     </r>
   </si>
   <si>
     <t>number of unique individuals</t>
   </si>
   <si>
-    <t>fill in in 'ProvenanceStatement' tab</t>
+    <t>Enter the value on the 'ProvenanceStatement' tab.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
fix(excel): apply 203 approved text corrections (#281)
</commit_message>
<xml_diff>
--- a/Documents/Health-RI_v2.1.0-for-FDP.xlsx
+++ b/Documents/Health-RI_v2.1.0-for-FDP.xlsx
@@ -78,7 +78,7 @@
     <t>Property URI</t>
   </si>
   <si>
-    <t>Controlled vocabluary (if applicable)</t>
+    <t>Controlled vocabulary (if applicable)</t>
   </si>
   <si>
     <t>Usage note</t>
@@ -138,16 +138,16 @@
     <t>custom:applicable_legislation</t>
   </si>
   <si>
-    <t>catalog</t>
-  </si>
-  <si>
-    <t>A catalog that is listed in the catalog.</t>
+    <t>catalogue</t>
+  </si>
+  <si>
+    <t>A catalogue that is listed in the catalogue.</t>
   </si>
   <si>
     <t>dcat:catalog</t>
   </si>
   <si>
-    <t>For certain research projects, multiple catalogs may need to be organized in a nested manner. This property serves to connect the different catalogs with each other.</t>
+    <t>For certain research projects, multiple catalogues may need to be organised in a nested manner. This property serves to connect the different catalogues with each other.</t>
   </si>
   <si>
     <t>dcat:Catalog</t>
@@ -165,7 +165,7 @@
     <t>contact point</t>
   </si>
   <si>
-    <t>Relevant contact information for the cataloged resource.</t>
+    <t>Relevant contact information for the catalogued resource.</t>
   </si>
   <si>
     <t>dcat:contactPoint</t>
@@ -178,7 +178,7 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t xml:space="preserve">This property points to a contact point that can answer questions about the dataset. Details on how to describe these are provided under class vcard:Kind.
+      <t xml:space="preserve">This property points to a contact point that can answer questions about the dataset. Details on how to describe these are provided under the vcard:Kind class.
 Whenever possible, use </t>
     </r>
     <r>
@@ -198,7 +198,7 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t xml:space="preserve"> (for example from a department) instead of the contact information of an individual.</t>
+      <t xml:space="preserve"> (for example, from a department) instead of the contact information of an individual.</t>
     </r>
   </si>
   <si>
@@ -214,7 +214,7 @@
     <t>custom:contact</t>
   </si>
   <si>
-    <t>fill in in 'Kind' tab</t>
+    <t>Enter the value on the 'Kind' tab.</t>
   </si>
   <si>
     <t>creator</t>
@@ -226,8 +226,8 @@
     <t>dct:creator</t>
   </si>
   <si>
-    <t>The creator is the entity responsible for making the resource. According to Dutch databank and copyright law, this is in most cases the organisation / employer bearing investment risk, instead of an individual (e.g. individual researcher). Therefore, in many cases, this might be the same Agent as the dct:publisher, being the organisation (not a department or subdivision of the organisation) where the catalogue was created.
-In case there are multiple (collaborating) organisations involved in data creation, all of them can be stated as dct:creator, as the model allows more than one creator.
+    <t>The creator is the entity responsible for making the resource. According to Dutch databank and copyright law, this is in most cases the organisation/employer bearing investment risk, instead of an individual (e.g. an individual researcher). Therefore, in many cases, this might be the same Agent as the dct:publisher: the organisation (not a department or subdivision of the organisation) where the catalogue was created.
+If there are multiple (collaborating) organisations involved in data creation, all of them can be stated as dct:creator, as the model allows more than one creator.
 Note that the Health-RI model diverges from DCAT-AP NL here, which reduces the maximum number of creators to 1. The Health-RI model allows the specification of multiple creators of a catalogue.</t>
   </si>
   <si>
@@ -237,19 +237,19 @@
     <t>custom:creator</t>
   </si>
   <si>
-    <t>fill in in 'Agent' tab</t>
+    <t>Enter the value on the 'Agent' tab.</t>
   </si>
   <si>
     <t>dataset</t>
   </si>
   <si>
-    <t>A dataset that is listed in the catalog.</t>
+    <t>A dataset that is listed in the catalogue.</t>
   </si>
   <si>
     <t>dcat:dataset</t>
   </si>
   <si>
-    <t>Each catalog contains one or more datasets. This property serves to link datasets to a catalogue. Therefore, a dataset is always contained inside a catalogue.</t>
+    <t>Each catalogue contains one or more datasets. This property serves to link datasets to a catalogue. Therefore, a dataset is always contained inside a catalogue.</t>
   </si>
   <si>
     <t>dcat:Dataset</t>
@@ -270,7 +270,7 @@
     <t>dct:description</t>
   </si>
   <si>
-    <t>Briefly describe the catalog and what it contains. You can repeat this in multiple languages.</t>
+    <t>Briefly describe the catalogue and what it contains. You can repeat this in multiple languages.</t>
   </si>
   <si>
     <t>rdfs:Literal</t>
@@ -291,7 +291,7 @@
     <t>EU Vocabularies Continents Named Authority List</t>
   </si>
   <si>
-    <t>The EU Vocabularies Name Authority Lists must be used for continents, countries and places that are in those lists; if a particular location is not in one of the mentioned Named Authority Lists, Geonames URIs must be used. For districts or neighbourhoods in NL, the Dutch vocab can be used.</t>
+    <t>The EU Vocabularies Named Authority Lists must be used for continents, countries and places that are in those lists; if a particular location is not in one of the mentioned Named Authority Lists, GeoNames URIs must be used. For districts or neighbourhoods in NL, the Dutch vocabulary can be used.</t>
   </si>
   <si>
     <t>dct:Location (IRI)</t>
@@ -306,7 +306,7 @@
     <t>EU Vocabularies Places Named Authority List</t>
   </si>
   <si>
-    <t>Geonames</t>
+    <t>GeoNames</t>
   </si>
   <si>
     <t>https://vocabs.cbs.nl/nl/</t>
@@ -322,10 +322,10 @@
   </si>
   <si>
     <t>Use this property to establish another catalogue in this catalogue.
-Note that deeply nested structures should be avoided, and can currently not be displayed in the National Health Data Catalogue.</t>
-  </si>
-  <si>
-    <t>If applicable, add URI to dcat:Catalog that is part of this catalogue</t>
+Note that deeply nested structures should be avoided, and cannot currently be displayed in the National Health Data Catalogue.</t>
+  </si>
+  <si>
+    <t>If applicable, add the URI of the dcat:Catalog that is part of this catalogue.</t>
   </si>
   <si>
     <t>home page</t>
@@ -410,7 +410,7 @@
     <t>dct:publisher</t>
   </si>
   <si>
-    <t>The organisation or individual that is holder of the intellectual property rights of a dataset. For more details about the publisher, see the class Agent. Example: Radboudumc.</t>
+    <t>The organisation or individual that is the holder of the intellectual property rights of a dataset. For more details about the publisher, see the class Agent. Example: Radboudumc.</t>
   </si>
   <si>
     <t>Adapted from v1</t>
@@ -449,13 +449,13 @@
     <t>service</t>
   </si>
   <si>
-    <t>A service that is listed in the catalog.</t>
+    <t>A service that is listed in the catalogue.</t>
   </si>
   <si>
     <t>dcat:service</t>
   </si>
   <si>
-    <t>Some datasets may have real-time Data Services (e.g., Beacon API counting individuals). IT teams should define the relationship between the catalog and the Data Service via this property. While crucial for interoperability, this property is not relevant for end-users to collect.</t>
+    <t>Some datasets may have real-time Data Services (e.g., Beacon API counting individuals). IT teams should define the relationship between the catalogue and the Data Service via this property. While crucial for interoperability, this property is not relevant for end users to collect.</t>
   </si>
   <si>
     <t>dcat:DataService</t>
@@ -488,7 +488,7 @@
     <t>dcat:themeTaxonomy</t>
   </si>
   <si>
-    <t>This property refers to a knowledge organisation system used to classify the Catalogue's Datasets. It must have at least the value NAL:data-theme as this is the mandatory controlled vocabulary for dcat:theme.</t>
+    <t>This property refers to a knowledge organisation system used to classify the Catalogue's Datasets. It must include at least the value NAL:data-theme as this is the mandatory controlled vocabulary for dcat:theme.</t>
   </si>
   <si>
     <t>skos:ConceptScheme</t>
@@ -503,7 +503,7 @@
     <t>dct:title</t>
   </si>
   <si>
-    <t>Provide a unique title for your catalog, which can be repeated in multiple languages. Example: Healthy Brain Study.</t>
+    <t>Provide a unique title for your catalogue, which can be repeated in multiple languages. Example: Healthy Brain Study.</t>
   </si>
   <si>
     <t>custom:purpose</t>
@@ -515,10 +515,10 @@
     <t>custom:retention_period</t>
   </si>
   <si>
-    <t>(issue on github)</t>
-  </si>
-  <si>
-    <t>issue on ckan github</t>
+    <t>(issue on GitHub)</t>
+  </si>
+  <si>
+    <t>issue on CKAN GitHub</t>
   </si>
   <si>
     <t>custom:status</t>
@@ -588,7 +588,7 @@
     <t>custom:analytics</t>
   </si>
   <si>
-    <t>If available, add URI to analytics distribution here</t>
+    <t>If available, add the URI for the analytics distribution here.</t>
   </si>
   <si>
     <t>code values</t>
@@ -609,7 +609,7 @@
     <t>coding system</t>
   </si>
   <si>
-    <t>Coding systems in use (ex: ICD-10-CM, DGRs, SNOMED=CT, ...)</t>
+    <t>Coding systems in use (e.g. ICD-10-CM, DGRs, SNOMED CT, ...)</t>
   </si>
   <si>
     <t>healthdcatap:hasCodingSystem</t>
@@ -636,15 +636,15 @@
     <t>custom:contact_</t>
   </si>
   <si>
-    <t>The creator (of the dataset) is the entity responsible for making the resource. According to Dutch databank and copyright law, this is in most cases the organisation / employer bearing investment risk, instead of an individual (e.g. individual researcher). Therefore, in many cases, this might be the same Agent as the dct:publisher, being the organisation (not a department or subdivision of the organisation) where the dataset was created.
-In case there are multiple (collaborating) organisations involved in data creation, all of them can be stated as dct:creator, as the model allows more than one creator.
+    <t>The creator (of the dataset) is the entity responsible for making the resource. According to Dutch databank and copyright law, this is in most cases the organisation/employer bearing investment risk, instead of an individual (e.g. an individual researcher). Therefore, in many cases, this might be the same Agent as the dct:publisher: the organisation (not a department or subdivision of the organisation) where the dataset was created.
+If there are multiple (collaborating) organisations involved in data creation, all of them can be stated as dct:creator, as the model allows more than one creator.
 In case you wish to credit other contributors to the dataset, you can use the prov:qualifiedAttribution property. This could be useful if you wish to indicate, for example, the funding organisation(s), collaborating organisation(s) or name specific individuals (e.g., principal investigator) involved in creating or managing the dataset.</t>
   </si>
   <si>
     <t>custom:creator_</t>
   </si>
   <si>
-    <t>Brief description of the dataset. You can repeat this property in multiple languages. Example: ''Collection of physiological data of Healthy Brain Study participants. This collection includes measurements via biowearables for heart rate, oxygenation, systolic and diastolic measures and stress levels.''</t>
+    <t>Brief description of the dataset. You can repeat this property in multiple languages. Example: ‘Collection of physiological data of Healthy Brain Study participants. This collection includes measurements via biowearables for heart rate, oxygenation, systolic and diastolic measures and stress levels.’</t>
   </si>
   <si>
     <t>distribution</t>
@@ -659,7 +659,7 @@
     <t>Metadata element used as a key link to the class Distribution.</t>
   </si>
   <si>
-    <t>fill in URI to dcat:Distribution</t>
+    <t>Enter the URI for dcat:Distribution.</t>
   </si>
   <si>
     <t>documentation</t>
@@ -671,7 +671,7 @@
     <t>foaf:page</t>
   </si>
   <si>
-    <t>The value of this property is the IRI directing to the web-page or document about the dataset.</t>
+    <t>The value of this property is the IRI pointing to the web page or document about the dataset.</t>
   </si>
   <si>
     <t>custom:documentation</t>
@@ -696,7 +696,7 @@
     <t>custom:frequency</t>
   </si>
   <si>
-    <t>The EU Vocabularies Name Authority Lists must be used for continents, countries and places that are in those lists; if a particular location is not in one of the mentioned Named Authority Lists, Geonames URIs must be used. For districts or neighbourhoods in NL, the Dutch vocab can be used. However, it might in many cases be desirable to keep the geographical coverage broader (e.g. indicating that NL is covered), to avoid exposing detailed information about subjects' locations.</t>
+    <t>The EU Vocabularies Named Authority Lists must be used for continents, countries and places that are in those lists; if a particular location is not in one of the mentioned Named Authority Lists, GeoNames URIs must be used. For districts or neighbourhoods in NL, the Dutch vocabulary can be used. However, it might in many cases be desirable to keep the geographical coverage broader (e.g. indicating that NL is covered), to avoid exposing detailed information about subjects' locations.</t>
   </si>
   <si>
     <t>has version</t>
@@ -708,7 +708,7 @@
     <t>dcat:hasVersion</t>
   </si>
   <si>
-    <t>Indicate the dataset which is the other version of the current dataset.</t>
+    <t>Indicate the dataset that is another version of the current dataset.</t>
   </si>
   <si>
     <t>custom:has_version</t>
@@ -739,7 +739,7 @@
   </si>
   <si>
     <t>Current status: Health-RI is currently working on a strategy for persistent identifiers for, among other things, datasets. Until a solid solution has been found, we propose the following temporary solution:
-If your data is published in a repository, fill in with the provided DOI (Example: https://doi.org/10.34894/ZLOYOJ). If not, use the identifier of the dataset as generated in the FAIR data point (FDP). Ensure that metadata is updated if your situation changes.</t>
+If your data is published in a repository, enter the provided DOI (Example: https://doi.org/10.34894/ZLOYOJ). If not, use the identifier of the dataset as generated in the FAIR data point (FDP). Ensure that metadata is updated if your situation changes.</t>
   </si>
   <si>
     <t>custom:alternate_identifier</t>
@@ -754,13 +754,13 @@
     <t>dcat:inSeries</t>
   </si>
   <si>
-    <t xml:space="preserve">This property points to which Dataset Series the Dataset is part of. </t>
+    <t xml:space="preserve">This property points to the Dataset Series of which the Dataset is part. </t>
   </si>
   <si>
     <t>dcat:DatasetSeries</t>
   </si>
   <si>
-    <t>If applicable, add URI to dataset series here</t>
+    <t>If applicable, add the URI for the dataset series here.</t>
   </si>
   <si>
     <t>is referenced by</t>
@@ -772,7 +772,7 @@
     <t>dct:isReferencedBy</t>
   </si>
   <si>
-    <t>The value of this property is the IRI of the doi to the publication or other related resource.
+    <t>The value of this property is the IRI of the DOI for the publication or other related resource.
 For example: https://doi.org/10.1186/s13690-021-00709-x</t>
   </si>
   <si>
@@ -884,7 +884,7 @@
     <t>adms:identifier</t>
   </si>
   <si>
-    <t>Examples for secondary identifiers are MAST/ADS, DataCite, DOI, EZID or W3ID (if not used for the original identifier). This property makes use of another, small class: adms:Identifier, where you provide the identifier and the name of the identifier schema (eg. DOI).</t>
+    <t>Examples of secondary identifiers include MAST/ADS, DataCite, DOI, EZID or W3ID (if not used for the original identifier). This property makes use of another small class: adms:Identifier, where you provide the identifier and the name of the identifier schema (e.g. DOI).</t>
   </si>
   <si>
     <t>adms:Identifier</t>
@@ -905,7 +905,7 @@
     <t>https://w3c.github.io/dpv/2.0/pd/</t>
   </si>
   <si>
-    <t>The different types of personal information that are collected in the dataset can be indicated with this property. Values can be picked from the dpv taxonomy (see controlled vocabulary column).
+    <t>The different types of personal information that are collected in the dataset can be indicated with this property. Values can be picked from the DPV taxonomy (see the Controlled vocabulary column).
 For example: dpv-pd:Gender</t>
   </si>
   <si>
@@ -921,13 +921,13 @@
     <t>healthdcatap:populationCoverage</t>
   </si>
   <si>
-    <t>This field is a free text description of the population covered in the dataset. For example, "Adults aged 18–65 diagnosed with type 2 diabetes in the Netherlands between 2015 and 2020".</t>
+    <t>This field is a free-text description of the population covered in the dataset. For example, "Adults aged 18–65 diagnosed with type 2 diabetes in the Netherlands between 2015 and 2020".</t>
   </si>
   <si>
     <t>custom:populatiion_coverage</t>
   </si>
   <si>
-    <t>This property identifies the organisation or individual responsible for making the dataset available. For datasets, this is typically the employer of the data creators. In simple cases, the dataset publisher may be the same as the catalog publisher. In more complex settings, such as when datasets come from multiple institutions within a consortium, the consortium should be listed as the publisher where possible. If no formal consortium can be specified, provide the information of the contributing organizations or individuals under dct:creator instead. For more details, refer to the Agent class.</t>
+    <t>This property identifies the organisation or individual responsible for making the dataset available. For datasets, this is typically the employer of the data creators. In simple cases, the dataset publisher may be the same as the catalogue publisher. In more complex settings, such as when datasets come from multiple institutions within a consortium, the consortium should be listed as the publisher where possible. If no formal consortium can be specified, provide information about the contributing organisations or individuals under dct:creator instead. For more details, refer to the Agent class.</t>
   </si>
   <si>
     <t>purpose</t>
@@ -1007,7 +1007,7 @@
     <t>prov:Attribution</t>
   </si>
   <si>
-    <t>fill in in 'Attribution' tab</t>
+    <t>Enter the value on the 'Attribution' tab.</t>
   </si>
   <si>
     <t>qualified relation</t>
@@ -1025,7 +1025,7 @@
     <t>dcat:Relationship</t>
   </si>
   <si>
-    <t>fill in in 'Relationship' tab</t>
+    <t>Enter the value on the 'Relationship' tab.</t>
   </si>
   <si>
     <t>quality annotation</t>
@@ -1043,7 +1043,7 @@
     <t>dqv:QualityCertificate</t>
   </si>
   <si>
-    <t>fill in in 'QualityCertificate' tab</t>
+    <t>Enter the value on the 'QualityCertificate' tab.</t>
   </si>
   <si>
     <r>
@@ -1098,13 +1098,13 @@
     <t>retention period</t>
   </si>
   <si>
-    <t>A temporal period which the dataset is available for secondary use.</t>
+    <t>A temporal period during which the dataset is available for secondary use.</t>
   </si>
   <si>
     <t>healthdcatap:retentionPeriod</t>
   </si>
   <si>
-    <t>fill in in 'Period of Time' tab</t>
+    <t>Enter the value on the 'PeriodOfTime' tab.</t>
   </si>
   <si>
     <t>sample</t>
@@ -1116,10 +1116,10 @@
     <t>adms:sample</t>
   </si>
   <si>
-    <t>This property makes use of the dcat:Distribution class to describe a sample distribution of the dataset, which can be anonymized or synthetic data, or the data dictionary provided in CSVW format. This is currently further developed by the TEHDAS2 program. More information can be found here: https://healthdcat-ap.github.io/#sample-distribution</t>
-  </si>
-  <si>
-    <t>If available, add URI to sample distribution here</t>
+    <t>This property makes use of the dcat:Distribution class to describe a sample distribution of the dataset, which can consist of anonymised or synthetic data, or a data dictionary provided in CSVW format. This is currently being further developed by the TEHDAS2 programme. More information can be found here: https://healthdcat-ap.github.io/#sample-distribution</t>
+  </si>
+  <si>
+    <t>If available, add the URI for the sample distribution here.</t>
   </si>
   <si>
     <t>source</t>
@@ -1134,7 +1134,7 @@
     <t>Indicate the dataset on which this described dataset is based.</t>
   </si>
   <si>
-    <t>If applicable, add URI to source dataset here</t>
+    <t>If applicable, add the URI for the source dataset here.</t>
   </si>
   <si>
     <t>status</t>
@@ -1165,7 +1165,7 @@
     <t>dcat:temporalResolution</t>
   </si>
   <si>
-    <t>If the dataset is a time-series, this should correspond to the spacing of items in the series. For other kinds of dataset, this property will usually indicate the smallest time difference between items in the dataset. The time period has to be provided in the xsd:duration format.</t>
+    <t>If the dataset is a time-series, this should correspond to the spacing of items in the series. For other kinds of datasets, this property will usually indicate the smallest time difference between items in the dataset. The time period has to be provided in the xsd:duration format.</t>
   </si>
   <si>
     <t>xsd:duration</t>
@@ -1219,7 +1219,7 @@
     <t>adms:versionNotes</t>
   </si>
   <si>
-    <t>Provide a short description of changes made to the dataset from the previous version.</t>
+    <t>Provide a short description of changes made to the dataset since the previous version.</t>
   </si>
   <si>
     <t>was generated by</t>
@@ -1284,7 +1284,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> of additional classes  (additional instances of Dataset, DatasetSeries, DataService or Catalogue)</t>
+      <t xml:space="preserve"> of additional classes (additional instances of Dataset, DatasetSeries, DataService or Catalogue).</t>
     </r>
   </si>
   <si>
@@ -1313,7 +1313,7 @@
 Wikidata: https://www.wikidata.org/wiki/Wikidata:Main_Page</t>
   </si>
   <si>
-    <t>Specify the entity (person or organization) by providing an identifier. We recommend using an ORCID identifier for a person or ROR identifier for an organization. Dutch government organizations are listed in TOOI. If these are not available, you can use ISNI, or Wikidata or any other identifier you may have. If you have multiple identifiers, you should provide them all.</t>
+    <t>Specify the entity (person or organisation) by providing an identifier. We recommend using an ORCID identifier for a person or a ROR identifier for an organisation. Dutch government organisations are listed in TOOI. If these are not available, you can use ISNI, Wikidata or any other identifier you may have. If you have multiple identifiers, you should provide them all.</t>
   </si>
   <si>
     <t>HRI v1</t>
@@ -1331,7 +1331,7 @@
     <t>foaf:name</t>
   </si>
   <si>
-    <t>This property refers to the given name of the entity. Example: Jane Doe (for a person) and Radboudumc (for an organization). This property can be repeated for different versions of the name (e.g. the name in different languages).</t>
+    <t>This property refers to the given name of the entity. Example: Jane Doe (for a person) and Radboudumc (for an organisation). This property can be repeated for different versions of the name (e.g. the name in different languages).</t>
   </si>
   <si>
     <t>_name</t>
@@ -1340,7 +1340,7 @@
     <t>publisher note</t>
   </si>
   <si>
-    <t>A description of the publisher activities.</t>
+    <t>A description of the publisher's activities.</t>
   </si>
   <si>
     <t>healthdcatap:publishernote</t>
@@ -1358,7 +1358,7 @@
     <t>https://raw.githubusercontent.com/SEMICeu/ADMS-AP/master/purl.org/ADMS_SKOS_v1.00.rdf</t>
   </si>
   <si>
-    <t>This property should be filled using ADMS vocabulary (http://purl.org/adms/publishertype/1.0)</t>
+    <t>This property should be filled using ADMS vocabulary (http://purl.org/adms/publishertype/1.0).</t>
   </si>
   <si>
     <t>_type</t>
@@ -1411,7 +1411,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> of additional classes ( (additional instances of Dataset, DatasetSeries, DataService or Catalogue)</t>
+      <t xml:space="preserve"> of additional classes (additional instances of Dataset, DatasetSeries, DataService or Catalogue).</t>
     </r>
   </si>
   <si>
@@ -1481,10 +1481,10 @@
     <t>resource:access_services</t>
   </si>
   <si>
-    <t>If applicable, fill in URI to dcat:DatasService</t>
-  </si>
-  <si>
-    <t>access url</t>
+    <t>If applicable, enter the URI for dcat:DataService.</t>
+  </si>
+  <si>
+    <t>access URL</t>
   </si>
   <si>
     <t>A URL of the resource that gives access to a distribution of the dataset. E.g., landing page, feed, SPARQL endpoint.</t>
@@ -1529,7 +1529,7 @@
     <t>spdx:checksum</t>
   </si>
   <si>
-    <t>The checksum is related to the downloadURL. This property makes use of the spdx:Checksum class, which itself has two properties to indicate checksum algorithm and checksum value (see Checksum class for further details).</t>
+    <t>The checksum is related to the downloadURL. This property makes use of the spdx:Checksum class, which itself has two properties to indicate the checksum algorithm and checksum value (see Checksum class for further details).</t>
   </si>
   <si>
     <t>spdx:Checksum</t>
@@ -1538,13 +1538,13 @@
     <t>resource:hash_algorithm/resource:hash_algorithm</t>
   </si>
   <si>
-    <t>fill in in 'Checksum' tab</t>
+    <t>Enter the value on the 'Checksum' tab.</t>
   </si>
   <si>
     <t>compression format</t>
   </si>
   <si>
-    <t>The compression format of the distribution in which the data is contained in a compressed form, e.g., to reduce the size of the downloadable file.</t>
+    <t>The compression format of the distribution in which the data is compressed, e.g., to reduce the size of the downloadable file.</t>
   </si>
   <si>
     <t>dcat:compressFormat</t>
@@ -1608,7 +1608,7 @@
   </si>
   <si>
     <r>
-      <t>Indicates the </t>
+      <t xml:space="preserve">Indicates the </t>
     </r>
     <r>
       <rPr>
@@ -1627,7 +1627,7 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t xml:space="preserve"> used in the Distribution, indicated with a value from the EU controlled vocabulary. Not all distributions might have a language, for example imaging data.
+      <t xml:space="preserve"> used in the Distribution, using a value from the EU controlled vocabulary. Not all distributions might have a language, for example imaging data.
 Note that here the Health-RI model diverges from DCAT-AP NL, which allows a maximum of 1 language per Distribution. The Health-RI model allows multiple languages in the same Distribution.</t>
     </r>
   </si>
@@ -1635,10 +1635,10 @@
     <t>resource:language</t>
   </si>
   <si>
-    <t>license</t>
-  </si>
-  <si>
-    <t>For public data, use a Creative Commons (CC) license (see Geonovum options in the Controlled Vocabulary column). For most National Health Data Catalogue distributions, where data is not public, use the 'not open' license from Geonovum and specify data reuse agreements in the dct:rights property.</t>
+    <t>licence</t>
+  </si>
+  <si>
+    <t>For public data, use a Creative Commons (CC) licence (see Geonovum options in the Controlled Vocabulary column). For most National Health Data Catalogue distributions, where data is not public, use the 'not open' licence from Geonovum and specify data reuse agreements in the dct:rights property.</t>
   </si>
   <si>
     <t>resource:license</t>
@@ -1662,7 +1662,7 @@
     <t>dcat:mediaType</t>
   </si>
   <si>
-    <t>Use the specified vocabularies, prioritizing IANA media types whenever possible. If unavailable, consider other ontologies, such as ZonMw generic terms, to describe the format.
+    <t>Use the specified vocabularies, prioritising IANA media types whenever possible. If unavailable, consider other ontologies, such as ZonMw generic terms, to describe the format.
 Example: https://www.iana.org/assignments/media-types/text/csv (for csv)
 If IANA media types do not sufficiently describe the format, use "format" to describe it in more detail.</t>
   </si>
@@ -1697,7 +1697,7 @@
     <t>healthdcatap:retentionperiod</t>
   </si>
   <si>
-    <t>fill in in 'Periof of Time' tab</t>
+    <t>Enter the value on the 'PeriodOfTime' tab.</t>
   </si>
   <si>
     <t>resource:rights</t>
@@ -1707,16 +1707,16 @@
 EU Vocabularies Distribution Status</t>
   </si>
   <si>
-    <t>It MUST take one of the values Completed, Deprecated, Under Development, Withdrawn from the provided controlled vocabulary.</t>
+    <t>It MUST take one of the following values from the provided controlled vocabulary: Completed, Deprecated, Under Development or Withdrawn.</t>
   </si>
   <si>
     <t>resource:status</t>
   </si>
   <si>
-    <t>If applicable, this property indicates the minimum time period resolvable in the dataset distribution, expressed in xsd:duration format (see for more information here: https://www.w3schools.com/xml/schema_dtypes_date.asp)</t>
-  </si>
-  <si>
-    <t>A title given to the distribution. e.g., Data Access Request of Healthy Brain study</t>
+    <t>If applicable, this property indicates the minimum time period resolvable in the dataset distribution, expressed in xsd:duration format (for more information, see: https://www.w3schools.com/xml/schema_dtypes_date.asp).</t>
+  </si>
+  <si>
+    <t>A title given to the distribution, e.g. Data Access Request for the Healthy Brain Study</t>
   </si>
   <si>
     <t>resource:name</t>
@@ -1734,7 +1734,7 @@
     <t>data_series::contact</t>
   </si>
   <si>
-    <t xml:space="preserve">Briefly describe the dataset series in the catalog. You can repeat this in multiple languages. </t>
+    <t xml:space="preserve">Briefly describe the dataset series in the catalogue. You can repeat this in multiple languages. </t>
   </si>
   <si>
     <t>data_series::modified</t>
@@ -1749,7 +1749,7 @@
     <t>This is not equal to the most recently modified dataset in the collection of the dataset series.</t>
   </si>
   <si>
-    <t xml:space="preserve">The publisher of the dataset series may not be the publisher of all datasets.  E.g. a digital archive could take over the publishing of older datasets in the series. </t>
+    <t xml:space="preserve">The publisher of the dataset series may not be the publisher of all datasets. For example, a digital archive could take over the publishing of older datasets in the series. </t>
   </si>
   <si>
     <t>data_series::publisher</t>
@@ -1761,7 +1761,7 @@
     <t>data_series:issued</t>
   </si>
   <si>
-    <t>When temporal coverage is a dimension in the dataset series then the temporal coverage of each dataset in the collection should be part of the temporal coverage. In that case, an open-ended value is recommended, e.g. after 2012.</t>
+    <t>When temporal coverage is a dimension in the dataset series, the temporal coverage of each dataset in the collection should be part of the series' temporal coverage. In that case, an open-ended value is recommended, e.g. after 2012.</t>
   </si>
   <si>
     <t>data_series::temporal</t>
@@ -1774,7 +1774,7 @@
   </si>
   <si>
     <r>
-      <t>Information that indicates whether the Dataset is publicly accessible, has access restrictions or is not public. This property is required to adopt one of the predefined values listed in the </t>
+      <t>Information that indicates whether the Dataset is publicly accessible, has access restrictions or is not public. This property must take one of the predefined values listed in the </t>
     </r>
     <r>
       <rPr>
@@ -1831,10 +1831,10 @@
     <t>access_service:description</t>
   </si>
   <si>
-    <t>end point description</t>
-  </si>
-  <si>
-    <t>A description of the services available via the end-points, including their operations, parameters etc.</t>
+    <t>endpoint description</t>
+  </si>
+  <si>
+    <t>A description of the services available via the endpoints, including their operations, parameters, etc.</t>
   </si>
   <si>
     <t>dcat:endpointDescription</t>
@@ -1846,7 +1846,7 @@
     <t>access_service:endpoint_description</t>
   </si>
   <si>
-    <t>end point URL</t>
+    <t>endpoint URL</t>
   </si>
   <si>
     <t>The root location or primary endpoint of the service (a Web-resolvable IRI).</t>
@@ -1870,22 +1870,22 @@
     <t>Provide a unique identifier for the data service. This could be a globally unique and persistent identifier, such as a DOI, URN, or UUID. If no persistent identifier is available, you may use the accessURL or endpointURL as the identifier, provided it is stable and unique to the service.</t>
   </si>
   <si>
-    <t>landing Page</t>
-  </si>
-  <si>
-    <t>A Web page that can be navigated to in a Web browser to gain access to the catalog, a dataset, its distributions and/or additional information.</t>
+    <t>landing page</t>
+  </si>
+  <si>
+    <t>A Web page that can be navigated to in a Web browser to gain access to the catalogue, a dataset, its distributions and/or additional information.</t>
   </si>
   <si>
     <t>dcat:landingPage</t>
   </si>
   <si>
-    <t>It is intended to point to a landing page at the original data service provider, not to a page on a site of a third party, such as an aggregator.</t>
+    <t>It is intended to point to a landing page at the original data service provider, not to a page on a third-party site, such as an aggregator.</t>
   </si>
   <si>
     <t>Indicates the natural language used in the data service, indicated with a value from the EU controlled vocabulary.</t>
   </si>
   <si>
-    <t>For public data, use a Creative Commons (CC) license (see Geonovum options in the Controlled Vocabulary column). For most National Health Data Catalogue data services, where data is not public, use the 'not open' license from Geonovum and specify data reuse agreements in the dct:rights property.</t>
+    <t>For public data, use a Creative Commons (CC) licence (see Geonovum options in the Controlled Vocabulary column). For most National Health Data Catalogue data services, where data is not public, use the 'not open' licence from Geonovum and specify data reuse agreements in the dct:rights property.</t>
   </si>
   <si>
     <t>access_service:license</t>
@@ -1894,10 +1894,10 @@
     <t>This property indicates the date of the last changes to the dataset, not the metadata record. An absent value may mean the resource hasn't changed since publication, the modification date is unknown, or the resource is continuously updated.</t>
   </si>
   <si>
-    <t>fill in in 'adms_Identifier' tab</t>
-  </si>
-  <si>
-    <t>The organization or individual responsible for making the data service available. In the context of data services, the publisher is typically the organization that manages or provides access to the service. For details, see the class Agent.</t>
+    <t>Enter the value on the 'adms_Identifier' tab.</t>
+  </si>
+  <si>
+    <t>The organisation or individual responsible for making the data service available. In the context of data services, the publisher is typically the organisation that manages or provides access to the service. For details, see the class Agent.</t>
   </si>
   <si>
     <t>serves dataset</t>
@@ -1915,13 +1915,13 @@
     <t>access_service:serves_dataset</t>
   </si>
   <si>
-    <t>fill in URI to dcat:Dataset that this data service serves</t>
+    <t>Enter the URI for the dcat:Dataset that this data service serves.</t>
   </si>
   <si>
     <t>This property should use a controlled vocabulary. In the Health Data Catalogue, most data services will use NAL:data-theme 'HEAL', but additional values from the same vocabulary are allowed.</t>
   </si>
   <si>
-    <t>Provide a unique title for your data service, which can be repeated in multiple languages. Example: Patient counts per available diagnosis</t>
+    <t>Provide a unique title for your data service, which can be repeated in multiple languages. Example: Patient counts per available diagnosis.</t>
   </si>
   <si>
     <t>access_service:title</t>
@@ -1959,7 +1959,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> of additional classes (additional instances of Dataset or DataService)</t>
+      <t xml:space="preserve"> of additional classes (additional instances of Dataset or DataService).</t>
     </r>
   </si>
   <si>
@@ -2045,7 +2045,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> of additional classes (additional instances of Catalogue, Dataset, Distribution or Dataset Series)</t>
+      <t xml:space="preserve"> of additional classes (additional instances of Catalogue, Dataset, Distribution or Dataset Series).</t>
     </r>
   </si>
   <si>
@@ -2067,13 +2067,13 @@
     <t>dcat:startDate</t>
   </si>
   <si>
-    <t>Value: qualified Attribution (Dataset A)</t>
-  </si>
-  <si>
-    <t>Value: qualified Attribution (Dataset B)</t>
-  </si>
-  <si>
-    <t>Value: qualified Attribution (Dataset C)</t>
+    <t>Value: qualified attribution (Dataset A)</t>
+  </si>
+  <si>
+    <t>Value: qualified attribution (Dataset B)</t>
+  </si>
+  <si>
+    <t>Value: qualified attribution (Dataset C)</t>
   </si>
   <si>
     <r>
@@ -2099,14 +2099,14 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> of additional classes (additional instances of Dataset)</t>
+      <t xml:space="preserve"> of additional classes (additional instances of Dataset).</t>
     </r>
   </si>
   <si>
     <t>agent</t>
   </si>
   <si>
-    <t>The prov:agent property references a prov:Agent which influenced a resource.</t>
+    <t>The prov:agent property references a prov:Agent that influenced a resource.</t>
   </si>
   <si>
     <t>prov:agent</t>
@@ -2131,16 +2131,16 @@
   <si>
     <t>Choose one of the roles as listed in the controlled vocabulary. Note that for HealthDCAT-AP, the list of roles might be extended in the future.
 Example: https://standards.iso.org/iso/19115/resources/Codelists/gml/CI_RoleCode.xml#processor
-Next to the CI_RoleCode, we also propose to use the CRediT Taxonomy to specify roles of contributors.</t>
-  </si>
-  <si>
-    <t>Value qualified Relation (Dataset A)</t>
-  </si>
-  <si>
-    <t>Value qualified Relation (Dataset B)</t>
-  </si>
-  <si>
-    <t>Value qualified Relation (Dataset C)</t>
+In addition to CI_RoleCode, we also propose to use the CRediT Taxonomy to specify roles of contributors.</t>
+  </si>
+  <si>
+    <t>Value: qualified relation (Dataset A)</t>
+  </si>
+  <si>
+    <t>Value: qualified relation (Dataset B)</t>
+  </si>
+  <si>
+    <t>Value: qualified relation (Dataset C)</t>
   </si>
   <si>
     <r>
@@ -2166,7 +2166,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t>of additional classes (additional instances of Dataset)</t>
+      <t>of additional classes (additional instances of Dataset).</t>
     </r>
   </si>
   <si>
@@ -2226,7 +2226,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> of additional classes (additional instances of Dataset)</t>
+      <t xml:space="preserve"> of additional classes (additional instances of Dataset).</t>
     </r>
   </si>
   <si>
@@ -2240,7 +2240,7 @@
   </si>
   <si>
     <t>This property has to be filled with the same value as the dct:identifier of the dataset described, in order to link the quality certificate to that dataset.
-See also example in HealthDCAT-AP: https://healthdcat-ap.github.io/#dqvhasqualityannotation</t>
+See also the example in HealthDCAT-AP: https://healthdcat-ap.github.io/#dqvhasqualityannotation</t>
   </si>
   <si>
     <t>body</t>
@@ -2345,7 +2345,7 @@
     <t xml:space="preserve">foaf:primaryTopic </t>
   </si>
   <si>
-    <t xml:space="preserve">A catalogue record will refer to one entity in a catalogue. This can be either a Dataset or a Data Service. To ensure an unambigous reading of the cardinality the range is set to Catalogued Resource. However it is not the intend with this range to require the explicit use of the class Catalogued Record. As abstract class, an subclass should be used. </t>
+    <t xml:space="preserve">A catalogue record will refer to one entity in a catalogue. This can be either a Dataset or a Data Service. To ensure an unambiguous reading of the cardinality, the range is set to Catalogued Resource. However, this range is not intended to require the explicit use of the class Catalogued Record. Since this is an abstract class, a subclass should be used. </t>
   </si>
   <si>
     <t xml:space="preserve">dcat:Resource </t>
@@ -2404,7 +2404,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> of additional classes (additional instances of Distribution)</t>
+      <t xml:space="preserve"> of additional classes (additional instances of Distribution).</t>
     </r>
   </si>
   <si>
@@ -2420,7 +2420,7 @@
     <t>https://spdx.org/rdf/terms/#d4e2129</t>
   </si>
   <si>
-    <t>Choose one member of the checksum algorithm members as indicated on the webpage linked in the Controlled Vocabulary column.</t>
+    <t>Choose one of the checksum algorithms as indicated on the webpage linked in the Controlled Vocabulary column.</t>
   </si>
   <si>
     <t>spdx:ChecksumAlgorithm (IRI)</t>
@@ -2440,13 +2440,13 @@
   <si>
     <t>It is preferred to provide a general email address of the appropriate institution or department instead of a personal email address, even if an individual is described with this instance of foaf:Agent.
 This protects their privacy and enables contact about the resource even after the individual has left the institution.
-The email address has to be provided starting with mailto: prefix.
+The email address must start with the mailto: prefix.
 For example: mailto:info@example.com</t>
   </si>
   <si>
     <t>It is preferred to provide a general email address of the appropriate institution or department instead of a personal email address, even if an individual is described with this instance of vcard:Kind.
 This protects their privacy and enables contact about the resource even after the individual has left the institution.
-The email address has to be provided starting with mailto: prefix.
+The email address must start with the mailto: prefix.
 For example: mailto:info@example.com</t>
   </si>
   <si>
@@ -2459,21 +2459,21 @@
   <si>
     <t>The ELI of the EHDS was published in March 2025 and can now be included as the applicable legislation mandating that the dataset has to be made public.
 For health datasets, the value must include the ELI of the EHDS Regulation (http://data.europa.eu/eli/reg/2025/327/oj).
-As multiple legislations may apply to the resource the maximum cardinality is not limited. Note that the relation with other legislations is complex and is being looked into by legal experts.
-While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property (also in Datasets) described the legal basis for initial collection and processing of (personal) data.</t>
-  </si>
-  <si>
-    <t>The legal basis can be provided as a value from the dpv taxonomy (see Controlled vocabulary column).
+As multiple pieces of legislation may apply to the resource, the maximum cardinality is not limited. Note that the relationship with other legislation is complex and is being looked into by legal experts.
+While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property (also in Datasets) describes the legal basis for initial collection and processing of (personal) data.</t>
+  </si>
+  <si>
+    <t>The legal basis can be provided as a value from the DPV taxonomy (see the Controlled vocabulary column).
 While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property describes the legal basis for initial collection and processing of (personal) data.
 This property should always be filled if the dataset contains personal data and the applicable legislation is GDPR.
-Example value for this property could be: dpv:Consent</t>
-  </si>
-  <si>
-    <t>One (or many) categories or sub-categories of the purposes can be chosen from the taxonomy provided by dpv (see controlled vocabulary column). Try to be as specific as possible.
-Example value could be: dpv:ResearchAndDevelopment.</t>
-  </si>
-  <si>
-    <t>Indicate with this property in case the Dataset is only available for secondary use for a specific period of time (e.g. due to data protection, contractual, or project constraints).
+An example value for this property could be dpv:Consent.</t>
+  </si>
+  <si>
+    <t>One or more categories or sub-categories of purposes can be chosen from the taxonomy provided by dpv (see the Controlled vocabulary column). Try to be as specific as possible.
+An example value could be dpv:ResearchAndDevelopment.</t>
+  </si>
+  <si>
+    <t>Use this property if the Dataset is only available for secondary use for a specific period of time (e.g. due to data protection, contractual, or project constraints).
 This property makes use of the class dct:PeriodOfTime, in which a start and end date can be provided.
 If the Dataset is available indefinitely, leave the property empty (cardinality is 0..1; it is only meaningful when a retention limit applies).
 If only a start is known, provide dcat:startDate only (open-ended interval, as allowed by dct:PeriodOfTime).
@@ -2576,7 +2576,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Display"/>
       </rPr>
-      <t>: The variables  have been added to the metadata model version 2.1 for testing purposes. For now it is not yet planned to be added to the national catalogue's front end.
+      <t>: The variables have been added to the metadata model version 2.1 for testing purposes. For now, their inclusion in the national catalogue's front end is not yet planned.
 Use this property to link a structured dataset to a CSVW TableGroup that documents its data variables, columns, or fields in a machine-readable way.</t>
     </r>
   </si>
@@ -2602,16 +2602,16 @@
     <t>Value: table 2</t>
   </si>
   <si>
-    <t>Add more columns if you need to describe additional instances of csvw:TableGroup</t>
+    <t>Add more columns if you need to describe additional instances of csvw:TableGroup.</t>
   </si>
   <si>
     <t>csvw:TableGroup</t>
   </si>
   <si>
-    <t>fill in in 'TableGroup' tab</t>
-  </si>
-  <si>
-    <t>fill in in 'TableGroup'  tab</t>
+    <t>Enter the value on the 'TableGroup' tab.</t>
+  </si>
+  <si>
+    <t>Enter the value on the 'TableGroup' tab.</t>
   </si>
   <si>
     <t>url</t>
@@ -2626,7 +2626,7 @@
     <t>Table title.</t>
   </si>
   <si>
-    <t xml:space="preserve">A keyword or tag describing the table.	</t>
+    <t xml:space="preserve">A keyword or tag describing the table.</t>
   </si>
   <si>
     <t>A variable (column) defines metadata about one field in the CSV file.</t>
@@ -2641,7 +2641,7 @@
     <t>csvw:column</t>
   </si>
   <si>
-    <t>The URL should be a valid IRI and should point to the CSV file (synthetic, anonymized representation of the real data) for this table.</t>
+    <t>The URL should be a valid IRI and should point to the CSV file (a synthetic, anonymised representation of the real data) for this table.</t>
   </si>
   <si>
     <t>Used to provide a human-readable title for the table. Can appear in multiple languages.</t>
@@ -2656,7 +2656,7 @@
     <t>csvw:Column</t>
   </si>
   <si>
-    <t>Add more columns if you need to describe additional instances of csvw:Table</t>
+    <t>Add more columns if you need to describe additional instances of csvw:Table.</t>
   </si>
   <si>
     <t>datatype</t>
@@ -2699,7 +2699,7 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Should match the </t>
+      <t xml:space="preserve">The value should match the </t>
     </r>
     <r>
       <rPr>
@@ -2719,7 +2719,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> of one of the CSVW types as defined in the Built-in datatypes from XML Schema. https://w3c.github.io/csvw/metadata/#datatypes Example: string, integer, boolean …</t>
+      <t xml:space="preserve"> of one of the CSVW types as defined in the Built-in datatypes from XML Schema. See: https://w3c.github.io/csvw/metadata/#datatypes
+Example: string, integer, boolean …</t>
     </r>
   </si>
   <si>
@@ -3179,7 +3180,7 @@
     <t>availability</t>
   </si>
   <si>
-    <t>An indication how long it is planned to keep the Distribution of the Dataset available.</t>
+    <t>An indication of how long it is planned to keep the Distribution of the Dataset available.</t>
   </si>
   <si>
     <t>dcatap:availability</t>
@@ -3209,7 +3210,7 @@
         <scheme val="major"/>
       </rPr>
       <t>: This property will be deprecated in the upcoming major release. It is recommended to indicate the planned availability of the distribution with the newly added Distribution.availability property. 
-Indicate with this property in case the Distribution is only available for secondary use for a specific period of time (e.g. due to data protection, contractual, or project constraints).
+Use this property if the Distribution is only available for secondary use for a specific period of time (e.g. due to data protection, contractual, or project constraints).
 This property makes use of the class dct:PeriodOfTime, in which a start and end date can be provided.
 If the Distribution is available indefinitely, leave the property empty (cardinality is 0..1; it is only meaningful when a retention limit applies).
 If only a start is known, provide dcat:startDate only (open-ended interval, as allowed by dct:PeriodOfTime).
@@ -3265,7 +3266,7 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> for identifiers of the Dataset, such as DOI; use </t>
+      <t xml:space="preserve"> for identifiers of the Dataset, such as a DOI; use </t>
     </r>
     <r>
       <rPr>
@@ -3327,7 +3328,7 @@
     </r>
   </si>
   <si>
-    <t>Information about how the data was collected, including methodologies, tools, and protocols used. This property can be repeated for different versions of the provenance (e.g. the provenance in different languages).
+    <t>Information about how the data was collected, including methodologies, tools, and protocols used. This property can be repeated for different versions of the provenance (e.g. in different languages).
 This is where the collection-method statements not captured by dedicated properties can be listed.</t>
   </si>
   <si>
@@ -3341,7 +3342,7 @@
   </si>
   <si>
     <t>Use this property to indicate which anatomical parts of the body are covered by the Dataset. Select the relevant anatomical structure from SNOMED CT. Multiple anatomical locations can be provided.
-Example: Dataset containing lung imaging data can use Lung structure (http://snomed.info/id/39607008).</t>
+Example: A dataset containing lung imaging data can use Lung structure (http://snomed.info/id/39607008).</t>
   </si>
   <si>
     <t>domain of the data</t>
@@ -3382,8 +3383,8 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t>: The use of wikidata URIs will be replaced with the terms from a controlled vocabulary in the next major release.
-This property provides information on which coding systems are in use in your dataset. For this, wikidata URIs must be used.</t>
+      <t>: The use of Wikidata URIs will be replaced with the terms from a controlled vocabulary in the next major release.
+This property provides information on which coding systems are in use in your dataset. For this, Wikidata URIs must be used.</t>
     </r>
   </si>
   <si>
@@ -3404,8 +3405,8 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t>: The use of wikidata URIs will be replaced with the terms from a controlled vocabulary in the next major release.
-If your data conforms to an established standard or specification, use this property to indicate which one. The wikidata URI of the specification must be used. Example: https://www.wikidata.org/wiki/Q19597236 for FHIR.</t>
+      <t>: The use of Wikidata URIs will be replaced with the terms from a controlled vocabulary in the next major release.
+If your data conforms to an established standard or specification, use this property to indicate which one. The Wikidata URI of the specification must be used. Example: https://www.wikidata.org/wiki/Q19597236 for FHIR.</t>
     </r>
   </si>
   <si>
@@ -3424,8 +3425,8 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Display"/>
       </rPr>
-      <t>: The use of wikidata URIs will be replaced with the terms from a controlled vocabulary in the next major release.
-This property is a structured way to tag the dataset with different health themes. This could include, for example, the specific disease the dataset is about. More details can be provided, if desirable, in the keywords property.  The wikidata URI of the health theme must be used here.</t>
+      <t>: The use of Wikidata URIs will be replaced with the terms from a controlled vocabulary in the next major release.
+This property is a structured way to tag the dataset with different health themes. This could include, for example, the specific disease the dataset is about. More details can be provided, if desirable, in the keywords property.  The Wikidata URI of the health theme must be used here.</t>
     </r>
   </si>
   <si>
@@ -3466,7 +3467,7 @@
     </r>
   </si>
   <si>
-    <t>A statement that concerns all rights not addressed in fields License or Access rights. In case of not open data (as specified in the dct:licence property), further agreements regarding data reuse (e.g. Data Transfer Agreement, DTA) should be stated in this property.
+    <t>A statement that concerns all rights not addressed in the Licence or Access rights fields. For data that is not open (as specified in the dct:license property), further agreements regarding data reuse (e.g. Data Transfer Agreement, DTA) should be stated in this property.
 The rights statement should be a free-text statement placed at a web-accessible location such that the value of this property is the IRI pointing to that statement.</t>
   </si>
   <si>
@@ -3490,7 +3491,7 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> be used to provide the email address of the Agent, specified using fully qualified mailto: URI scheme RFC6068. The email </t>
+      <t xml:space="preserve"> be used to provide the email address of the Agent, specified using the fully qualified mailto: URI scheme defined in RFC 6068. The email </t>
     </r>
     <r>
       <rPr>
@@ -3542,8 +3543,8 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t>: The use of wikidata URIs will be replaced with free text in the next major release.
-Inside this property, you can provide the coding system of the dataset in the form of wikidata URI (example: https://www.wikidata.org/entity/P494 for ICD-10 ID) and the URI of the value that describes the dataset (example: https://icd.who.int/browse10/2019/en#/Y59.0 for viral vaccines)</t>
+      <t>: The use of Wikidata URIs will be replaced with free text in the next major release.
+Inside this property, you can provide the coding system of the dataset in the form of a Wikidata URI (example: https://www.wikidata.org/entity/P494 for ICD-10 ID) and the URI of the value that describes the dataset (example: https://icd.who.int/browse10/2019/en#/Y59.0 for viral vaccines).</t>
     </r>
   </si>
   <si>
@@ -3563,19 +3564,19 @@
     <t>rdfs:label</t>
   </si>
   <si>
-    <t>In this context the definition should be considered as: A textual statement describing the provenance of the Dataset, including information about its origin, history, or activities involved in its creation or modification.</t>
+    <t>In this context, the definition should be considered as: A textual statement describing the provenance of the Dataset, including information about its origin, history, or activities involved in its creation or modification.</t>
   </si>
   <si>
     <t>dct:ProvenanceStatement</t>
   </si>
   <si>
-    <t>Provide a short textual statement describing the provenance of the Dataset, such as its origin, how it was created or collected, or any relevant processing or transformations it has undergone. This statement should describe the provenance of the Dataset as a whole and be provided as free text.  You can repeat this property in multiple languages</t>
+    <t>Provide a short textual statement describing the provenance of the Dataset, such as its origin, how it was created or collected, or any relevant processing or transformations it has undergone. This statement should describe the provenance of the Dataset as a whole and be provided as free text. You can repeat this property in multiple languages.</t>
   </si>
   <si>
     <t>Value: activity (Dataset A)</t>
   </si>
   <si>
-    <t>Value:activity (Dataset B)</t>
+    <t>Value: activity (Dataset B)</t>
   </si>
   <si>
     <t>Value: activity (Dataset C)</t>
@@ -3590,7 +3591,7 @@
     <t>Value: provenance (Dataset 2)</t>
   </si>
   <si>
-    <t>Add more columns if you need to describe additional instances of dct:ProvenanceStatement for provenance of additional classes (additional instances of Dataset)</t>
+    <t>Add more columns if you need to describe additional instances of dct:ProvenanceStatement for provenance of additional classes (additional instances of Dataset).</t>
   </si>
   <si>
     <t>ProvenanceStatement</t>
@@ -3610,7 +3611,8 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Select data domain(s) from the predefined value list, available at this link: https://github.com/Health-RI/health-ri-metadata/blob/v2.1-changes/Formalisation(shacl)/Core/ValueLists/edam-has-topic.tsv </t>
+      <t xml:space="preserve">Select data domain(s) from the predefined value list, available at this link: https://github.com/Health-RI/health-ri-metadata/blob/v2.1-changes/Formalisation(shacl)/Core/ValueLists/edam-has-topic.tsv
+</t>
     </r>
     <r>
       <rPr>
@@ -3629,7 +3631,7 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t>: This is a temporary location and it will change with the release . 
+      <t>: This is a temporary location and it will change with the release. 
 A data domain refers to the broader scientific or health-related area covered by the Dataset. Select the domain that best represents the Dataset as a whole, rather than a specific data element within it. If the dataset contains data from more than one domain, you can select multiple.
 See the property "measurement technique" for more information about the technique(s) used to generate the data in the Dataset.</t>
     </r>
@@ -3673,8 +3675,9 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Select a suitable value or suitable values from the value list to indicate the technique(s) used to generate data in the dataset.
-The value list is  available at this link: https://github.com/Health-RI/health-ri-metadata/blob/v2.1-changes/Formalisation(shacl)/Core/ValueLists/schema-measurement-technique.tsv </t>
+      <t xml:space="preserve">Select one or more suitable values from the value list to indicate the technique(s) used to generate data in the dataset.
+The value list is available at this link: https://github.com/Health-RI/health-ri-metadata/blob/v2.1-changes/Formalisation(shacl)/Core/ValueLists/schema-measurement-technique.tsv
+</t>
     </r>
     <r>
       <rPr>
@@ -3693,14 +3696,14 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t xml:space="preserve">: This is a temporary location and it will change with the next release . </t>
+      <t xml:space="preserve">: This is a temporary location and it will change with the next release. </t>
     </r>
   </si>
   <si>
     <t>number of unique individuals</t>
   </si>
   <si>
-    <t>fill in in 'ProvenanceStatement' tab</t>
+    <t>Enter the value on the 'ProvenanceStatement' tab.</t>
   </si>
 </sst>
 </file>

</xml_diff>